<commit_message>
Aggiunge 13 nuovi fondi (totale 31)
Nuove categorie: America Latina, Energia, Europa Emergente,
Mercati Emergenti, Europa/Africa/ME + altri Materie Prime.
Tutti inseriti a Livello 3 (Universe/watchlist).

Co-Authored-By: Claude Opus 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fondi_monitoraggio.xlsx
+++ b/fondi_monitoraggio.xlsx
@@ -376,7 +376,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K19"/>
+  <dimension ref="A1:K32"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="8.710000000000001" customWidth="1" style="7" min="1" max="1"/>
@@ -1039,18 +1039,396 @@
       <c r="J19" s="1" t="n"/>
       <c r="K19" s="1" t="n"/>
     </row>
-    <row r="21" ht="15.75" customHeight="1" s="7"/>
-    <row r="22" ht="15.75" customHeight="1" s="7"/>
-    <row r="23" ht="15.75" customHeight="1" s="7"/>
-    <row r="24" ht="15.75" customHeight="1" s="7"/>
-    <row r="25" ht="15.75" customHeight="1" s="7"/>
-    <row r="26" ht="15.75" customHeight="1" s="7"/>
-    <row r="27" ht="15.75" customHeight="1" s="7"/>
-    <row r="28" ht="15.75" customHeight="1" s="7"/>
-    <row r="29" ht="15.75" customHeight="1" s="7"/>
-    <row r="30" ht="15.75" customHeight="1" s="7"/>
-    <row r="31" ht="15.75" customHeight="1" s="7"/>
-    <row r="32" ht="15.75" customHeight="1" s="7"/>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>3</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>LU0552029661</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>AMUNDI FUNDS LATIN AMERICA EQUITY - G EUR (C)</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Amundi</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Azionari America Latina</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="15.75" customHeight="1" s="7">
+      <c r="A21" t="n">
+        <v>3</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>LU1213835942</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Fidelity Funds - Latin America Fund A-ACC-EUR</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Fidelity</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Azionari America Latina</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="15.75" customHeight="1" s="7">
+      <c r="A22" t="n">
+        <v>3</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>LU0309468808</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Nordea-1 Latin American Eq BP Acc</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Nordea</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Azionari America Latina</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="15.75" customHeight="1" s="7">
+      <c r="A23" t="n">
+        <v>3</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>LU0522352862</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>JPMorgan Funds - JPM Latin America Equity D (acc) - EUR</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>JPMorgan</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Azionari America Latina</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="15.75" customHeight="1" s="7">
+      <c r="A24" t="n">
+        <v>3</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>LU0326425351</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>BlackRock Global Funds - World Mining Hedged E2 EUR</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>BlackRock</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Azionari Materie Prime</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="15.75" customHeight="1" s="7">
+      <c r="A25" t="n">
+        <v>3</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>LU0172157363</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>BGF World Mining Euro E</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>BlackRock</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Azionari Materie Prime</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="15.75" customHeight="1" s="7">
+      <c r="A26" t="n">
+        <v>3</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>LU0106817157</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Schroder ISF Emerg Eur A Acc</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Schroders</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Azionari Europa Emergente</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="15.75" customHeight="1" s="7">
+      <c r="A27" t="n">
+        <v>3</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>LU0326422507</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>BlackRock Global Funds - World Energy Hedged E2 EUR</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>BlackRock</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Azionari Energia</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="15.75" customHeight="1" s="7">
+      <c r="A28" t="n">
+        <v>3</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>LU0171304552</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>BGF World Energy Euro E</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>BlackRock</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Azionari Energia</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="15.75" customHeight="1" s="7">
+      <c r="A29" t="n">
+        <v>3</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>LU0056052961</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Candriam Equities L Emerging Markets C EUR Acc</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Candriam</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Azionari Mercati Emergenti</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="15.75" customHeight="1" s="7">
+      <c r="A30" t="n">
+        <v>3</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>LU1882448316</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Amundi Fds - Emerging Europe Middle East and Africa - cl E2 Eur C</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Amundi</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Azionari Europa/Africa/ME</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="15.75" customHeight="1" s="7">
+      <c r="A31" t="n">
+        <v>3</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>LU0303816028</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Fidelity Funds - Emerging Europe, Middle East and Africa A Euro</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Fidelity</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Azionari Europa/Africa/ME</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="15.75" customHeight="1" s="7">
+      <c r="A32" t="n">
+        <v>3</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>LU0307839646</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Fidelity Funds - Emerging Markets A Euro</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Fidelity</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Azionari Mercati Emergenti</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
     <row r="33" ht="15.75" customHeight="1" s="7"/>
     <row r="34" ht="15.75" customHeight="1" s="7"/>
     <row r="35" ht="15.75" customHeight="1" s="7"/>

</xml_diff>

<commit_message>
Aggiunti 32 fondi curati + fix detect_asset_type per Monetari e EM bonds
Nuovi fondi per settori mancanti (Healthcare, Finanziari, Infrastrutture,
Consumer) e aree geografiche (USA, Europa, Giappone, Asia, Cina, India,
Globali) + obbligazionari HY/EM/Globali + monetari.
Fix: Monetari ora rilevati come profilo 'bond', EM bonds come 'bond_hy'.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fondi_monitoraggio.xlsx
+++ b/fondi_monitoraggio.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:K32"/>
+  <dimension ref="A1:K64"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43359375" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="8.710000000000001" customWidth="1" style="7" min="1" max="1"/>
@@ -1936,38 +1936,1126 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="15.75" customHeight="1" s="8"/>
-    <row r="34" ht="15.75" customHeight="1" s="8"/>
-    <row r="35" ht="15.75" customHeight="1" s="8"/>
-    <row r="36" ht="15.75" customHeight="1" s="8"/>
-    <row r="37" ht="15.75" customHeight="1" s="8"/>
-    <row r="38" ht="15.75" customHeight="1" s="8"/>
-    <row r="39" ht="15.75" customHeight="1" s="8"/>
-    <row r="40" ht="15.75" customHeight="1" s="8"/>
-    <row r="41" ht="15.75" customHeight="1" s="8"/>
-    <row r="42" ht="15.75" customHeight="1" s="8"/>
-    <row r="43" ht="15.75" customHeight="1" s="8"/>
-    <row r="44" ht="15.75" customHeight="1" s="8"/>
-    <row r="45" ht="15.75" customHeight="1" s="8"/>
-    <row r="46" ht="15.75" customHeight="1" s="8"/>
-    <row r="47" ht="15.75" customHeight="1" s="8"/>
-    <row r="48" ht="15.75" customHeight="1" s="8"/>
-    <row r="49" ht="15.75" customHeight="1" s="8"/>
-    <row r="50" ht="15.75" customHeight="1" s="8"/>
-    <row r="51" ht="15.75" customHeight="1" s="8"/>
-    <row r="52" ht="15.75" customHeight="1" s="8"/>
-    <row r="53" ht="15.75" customHeight="1" s="8"/>
-    <row r="54" ht="15.75" customHeight="1" s="8"/>
-    <row r="55" ht="15.75" customHeight="1" s="8"/>
-    <row r="56" ht="15.75" customHeight="1" s="8"/>
-    <row r="57" ht="15.75" customHeight="1" s="8"/>
-    <row r="58" ht="15.75" customHeight="1" s="8"/>
-    <row r="59" ht="15.75" customHeight="1" s="8"/>
-    <row r="60" ht="15.75" customHeight="1" s="8"/>
-    <row r="61" ht="15.75" customHeight="1" s="8"/>
-    <row r="62" ht="15.75" customHeight="1" s="8"/>
-    <row r="63" ht="15.75" customHeight="1" s="8"/>
-    <row r="64" ht="15.75" customHeight="1" s="8"/>
+    <row r="33" ht="15.75" customHeight="1" s="8">
+      <c r="A33" t="n">
+        <v>3</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>LU0114720955</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Fidelity Funds - Global Health Care A EUR</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Fidelity</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Azionari Salute/Pharma</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="15.75" customHeight="1" s="8">
+      <c r="A34" t="n">
+        <v>3</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>LU0329630130</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>JPMorgan Funds - Global Healthcare A EUR</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>JPMorgan</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Azionari Salute/Pharma</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="15.75" customHeight="1" s="8">
+      <c r="A35" t="n">
+        <v>3</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>LU0329455071</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Candriam Equities L Oncology Impact C EUR</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Candriam</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Azionari Salute/Pharma</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="15.75" customHeight="1" s="8">
+      <c r="A36" t="n">
+        <v>3</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>LU0473185139</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Fidelity Funds - Global Financial Services A EUR</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Fidelity</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Azionari Finanziari</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="15.75" customHeight="1" s="8">
+      <c r="A37" t="n">
+        <v>3</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>LU0210527791</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>JPMorgan Funds - Europe Equity A EUR</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>JPMorgan</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Azionari Finanziari</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="15.75" customHeight="1" s="8">
+      <c r="A38" t="n">
+        <v>3</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>LU0363470070</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>DWS Invest Global Infrastructure LC</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>DWS</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Azionari Infrastrutture</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="15.75" customHeight="1" s="8">
+      <c r="A39" t="n">
+        <v>3</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>LU0187079347</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Invesco Global Consumer Trends A EUR</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Invesco</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Azionari Consumi/Lusso</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="15.75" customHeight="1" s="8">
+      <c r="A40" t="n">
+        <v>3</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>LU0640476718</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Fidelity Funds - Sustainable Consumer Brands A EUR</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Fidelity</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Azionari Consumi/Lusso</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="15.75" customHeight="1" s="8">
+      <c r="A41" t="n">
+        <v>3</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>LU0210534433</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>JPMorgan Funds - US Growth A EUR</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>JPMorgan</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Azionari USA</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="15.75" customHeight="1" s="8">
+      <c r="A42" t="n">
+        <v>3</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>LU0069450822</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Fidelity Funds - America Fund A EUR</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Fidelity</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Azionari USA</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="15.75" customHeight="1" s="8">
+      <c r="A43" t="n">
+        <v>3</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>LU1213835603</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Amundi Fds - Pioneer US Equity Fundamental Growth A EUR C</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Amundi</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Azionari USA</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="15.75" customHeight="1" s="8">
+      <c r="A44" t="n">
+        <v>3</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>LU0210073469</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>JPMorgan Funds - Europe Dynamic A EUR</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>JPMorgan</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Azionari Europa</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="15.75" customHeight="1" s="8">
+      <c r="A45" t="n">
+        <v>3</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>LU0346388373</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Nordea 1 - European Stars Equity BP EUR</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Nordea</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Azionari Europa</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="15.75" customHeight="1" s="8">
+      <c r="A46" t="n">
+        <v>3</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>LU0119750205</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Fidelity Funds - European Growth A EUR</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Fidelity</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Azionari Europa</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="15.75" customHeight="1" s="8">
+      <c r="A47" t="n">
+        <v>3</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>LU0161332480</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>JPMorgan Funds - Japan Equity A EUR</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>JPMorgan</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Azionari Giappone</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="15.75" customHeight="1" s="8">
+      <c r="A48" t="n">
+        <v>3</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>LU0413542167</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Schroders ISF Japanese Equity A EUR Hdg</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Schroders</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Azionari Giappone</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="15.75" customHeight="1" s="8">
+      <c r="A49" t="n">
+        <v>3</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>LU0210526066</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>JPMorgan Funds - Pacific Equity A EUR</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>JPMorgan</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Azionari Asia Pacifico</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="15.75" customHeight="1" s="8">
+      <c r="A50" t="n">
+        <v>3</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>LU0048597586</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Fidelity Funds - Asia Focus A EUR</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Fidelity</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Azionari Asia Pacifico</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="15.75" customHeight="1" s="8">
+      <c r="A51" t="n">
+        <v>3</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>LU0210526579</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>JPMorgan Funds - China A EUR</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>JPMorgan</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Azionari Cina</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="15.75" customHeight="1" s="8">
+      <c r="A52" t="n">
+        <v>3</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>LU1213836676</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Amundi Fds - China Equity A EUR C</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Amundi</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Azionari Cina</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="15.75" customHeight="1" s="8">
+      <c r="A53" t="n">
+        <v>3</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>LU0333810181</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>JPMorgan Funds - India A EUR</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>JPMorgan</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Azionari India</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="15.75" customHeight="1" s="8">
+      <c r="A54" t="n">
+        <v>3</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>LU0210534516</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>JPMorgan Funds - Global Select Equity A EUR</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>JPMorgan</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Azionari Globali</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="15.75" customHeight="1" s="8">
+      <c r="A55" t="n">
+        <v>3</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>LU0605515377</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Nordea 1 - Global Stars Equity BP EUR</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Nordea</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Azionari Globali</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="15.75" customHeight="1" s="8">
+      <c r="A56" t="n">
+        <v>3</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>LU0210531934</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>JPMorgan Funds - Europe High Yield Bond A EUR</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>JPMorgan</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Obbligazionari High Yield</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="15.75" customHeight="1" s="8">
+      <c r="A57" t="n">
+        <v>3</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>LU0159052710</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Candriam Bonds Euro High Yield C EUR</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Candriam</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Obbligazionari High Yield</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="15.75" customHeight="1" s="8">
+      <c r="A58" t="n">
+        <v>3</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>LU0155953517</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Fidelity Funds - European High Yield A EUR</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Fidelity</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Obbligazionari High Yield</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="15.75" customHeight="1" s="8">
+      <c r="A59" t="n">
+        <v>3</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>LU0522351971</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>JPMorgan Funds - Emerging Markets Debt A EUR Hdg</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>JPMorgan</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Obbligazionari Mercati Emergenti</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="15.75" customHeight="1" s="8">
+      <c r="A60" t="n">
+        <v>3</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>LU0238205289</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Amundi Fds - Emerging Markets Bond A EUR C</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Amundi</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Obbligazionari Mercati Emergenti</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="15.75" customHeight="1" s="8">
+      <c r="A61" t="n">
+        <v>3</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>LU0210531850</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>JPMorgan Funds - Global Bond Opportunities A EUR Hdg</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>JPMorgan</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Obbligazionari Globali</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="15.75" customHeight="1" s="8">
+      <c r="A62" t="n">
+        <v>3</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>LU0168060498</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Nordea 1 - European Covered Bond BP EUR</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Nordea</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Obbligazionari Globali</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="15.75" customHeight="1" s="8">
+      <c r="A63" t="n">
+        <v>3</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>FR0010510800</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Amundi Fds - Euro Government Bond A EUR C</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Amundi</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Monetari Euro</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="15.75" customHeight="1" s="8">
+      <c r="A64" t="n">
+        <v>3</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>LU0568621618</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>JPMorgan Funds - Euro Government Liquidity A EUR</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>JPMorgan</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Monetari Euro</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+    </row>
     <row r="65" ht="15.75" customHeight="1" s="8"/>
     <row r="66" ht="15.75" customHeight="1" s="8"/>
     <row r="67" ht="15.75" customHeight="1" s="8"/>

</xml_diff>

<commit_message>
Fix: migra email da Gmail SMTP a Resend API (HTTPS)
Railway blocca le connessioni SMTP in uscita (porta 587).
Resend usa HTTPS → non bloccato da Railway.
- alerts.py: rimosso smtplib, aggiunto resend SDK
- requirements.txt: aggiunto resend>=2.0.0
- .env.template: RESEND_API_KEY sostituisce EMAIL_PASSWORD

Da fare su Railway: aggiungere variabile RESEND_API_KEY
e aggiornare MONITOR_HOUR=17, MONITOR_DAYS=1-5

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fondi_monitoraggio.xlsx
+++ b/fondi_monitoraggio.xlsx
@@ -538,7 +538,7 @@
         <v>291.67</v>
       </c>
       <c r="H2" t="n">
-        <v>286.101</v>
+        <v>288.1415</v>
       </c>
       <c r="I2" t="n">
         <v>61.92</v>
@@ -550,7 +550,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -587,7 +587,7 @@
         <v>369.06</v>
       </c>
       <c r="H3" t="n">
-        <v>346.281</v>
+        <v>352.627</v>
       </c>
       <c r="I3" t="n">
         <v>63.63</v>
@@ -599,7 +599,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -636,7 +636,7 @@
         <v>315.41</v>
       </c>
       <c r="H4" t="n">
-        <v>295.988</v>
+        <v>301.397</v>
       </c>
       <c r="I4" t="n">
         <v>65.02</v>
@@ -648,7 +648,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -685,7 +685,7 @@
         <v>18.95</v>
       </c>
       <c r="H5" t="n">
-        <v>18.301</v>
+        <v>18.4835</v>
       </c>
       <c r="I5" t="n">
         <v>65.36</v>
@@ -697,7 +697,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -734,7 +734,7 @@
         <v>19.99</v>
       </c>
       <c r="H6" t="n">
-        <v>20.076</v>
+        <v>20.0685</v>
       </c>
       <c r="I6" t="n">
         <v>42.22</v>
@@ -746,7 +746,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -795,7 +795,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -832,19 +832,19 @@
         <v>125.74</v>
       </c>
       <c r="H8" t="n">
-        <v>125.5842</v>
+        <v>125.6295</v>
       </c>
       <c r="I8" t="n">
         <v>79.52</v>
       </c>
-      <c r="J8" s="1" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>SELL</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -881,19 +881,19 @@
         <v>94.98</v>
       </c>
       <c r="H9" t="n">
-        <v>94.85299999999999</v>
+        <v>94.8905</v>
       </c>
       <c r="I9" t="n">
         <v>82.16</v>
       </c>
-      <c r="J9" s="1" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>SELL</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -930,7 +930,7 @@
         <v>17.13</v>
       </c>
       <c r="H10" t="n">
-        <v>17.1214</v>
+        <v>17.1255</v>
       </c>
       <c r="I10" t="n">
         <v>69.59999999999999</v>
@@ -942,7 +942,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -979,19 +979,19 @@
         <v>7.68</v>
       </c>
       <c r="H11" t="n">
-        <v>7.6715</v>
+        <v>7.6745</v>
       </c>
       <c r="I11" t="n">
         <v>68.19</v>
       </c>
-      <c r="J11" s="1" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>SELL</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -1028,7 +1028,7 @@
         <v>10.83</v>
       </c>
       <c r="H12" t="n">
-        <v>10.8215</v>
+        <v>10.825</v>
       </c>
       <c r="I12" t="n">
         <v>74.66</v>
@@ -1040,7 +1040,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -1077,7 +1077,7 @@
         <v>123.08</v>
       </c>
       <c r="H13" t="n">
-        <v>122.852</v>
+        <v>122.9215</v>
       </c>
       <c r="I13" t="n">
         <v>62.65</v>
@@ -1089,7 +1089,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -1126,7 +1126,7 @@
         <v>149.61</v>
       </c>
       <c r="H14" t="n">
-        <v>149.526</v>
+        <v>149.544</v>
       </c>
       <c r="I14" t="n">
         <v>54.78</v>
@@ -1138,7 +1138,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -1175,7 +1175,7 @@
         <v>56.76</v>
       </c>
       <c r="H15" t="n">
-        <v>57.501</v>
+        <v>57.3735</v>
       </c>
       <c r="I15" t="n">
         <v>37.35</v>
@@ -1187,7 +1187,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -1224,7 +1224,7 @@
         <v>22.51</v>
       </c>
       <c r="H16" t="n">
-        <v>22.271</v>
+        <v>22.367</v>
       </c>
       <c r="I16" t="n">
         <v>52.57</v>
@@ -1236,7 +1236,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -1285,7 +1285,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -1322,7 +1322,7 @@
         <v>71.75</v>
       </c>
       <c r="H18" t="n">
-        <v>72.699</v>
+        <v>72.5335</v>
       </c>
       <c r="I18" t="n">
         <v>37.19</v>
@@ -1334,7 +1334,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -1371,7 +1371,7 @@
         <v>15.17</v>
       </c>
       <c r="H19" t="n">
-        <v>14.9555</v>
+        <v>15.031</v>
       </c>
       <c r="I19" t="n">
         <v>63.25</v>
@@ -1383,7 +1383,7 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -1420,7 +1420,7 @@
         <v>20.1</v>
       </c>
       <c r="H20" t="n">
-        <v>19.7345</v>
+        <v>19.8125</v>
       </c>
       <c r="I20" t="n">
         <v>67.68000000000001</v>
@@ -1432,7 +1432,7 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -1469,19 +1469,19 @@
         <v>116.14</v>
       </c>
       <c r="H21" t="n">
-        <v>113.71</v>
+        <v>114.377</v>
       </c>
       <c r="I21" t="n">
         <v>67.59</v>
       </c>
-      <c r="J21" s="2" t="inlineStr">
-        <is>
-          <t>BUY</t>
+      <c r="J21" s="1" t="inlineStr">
+        <is>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -1530,7 +1530,7 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -1567,7 +1567,7 @@
         <v>32.65</v>
       </c>
       <c r="H23" t="n">
-        <v>32.5763</v>
+        <v>32.583</v>
       </c>
       <c r="I23" t="n">
         <v>56.51</v>
@@ -1579,7 +1579,7 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -1628,7 +1628,7 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -1665,19 +1665,19 @@
         <v>1382.77</v>
       </c>
       <c r="H25" t="n">
-        <v>1334.846</v>
+        <v>1345.8625</v>
       </c>
       <c r="I25" t="n">
         <v>68.48</v>
       </c>
-      <c r="J25" s="1" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -1726,7 +1726,7 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -1763,7 +1763,7 @@
         <v>19.18</v>
       </c>
       <c r="H27" t="n">
-        <v>18.847</v>
+        <v>18.942</v>
       </c>
       <c r="I27" t="n">
         <v>66</v>
@@ -1775,7 +1775,7 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -1812,7 +1812,7 @@
         <v>21.94</v>
       </c>
       <c r="H28" t="n">
-        <v>21.5235</v>
+        <v>21.6945</v>
       </c>
       <c r="I28" t="n">
         <v>68.38</v>
@@ -1824,7 +1824,7 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -1861,7 +1861,7 @@
         <v>62.45</v>
       </c>
       <c r="H29" t="n">
-        <v>62.1505</v>
+        <v>62.2185</v>
       </c>
       <c r="I29" t="n">
         <v>50.07</v>
@@ -1873,7 +1873,7 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -1922,7 +1922,7 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -1971,7 +1971,7 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -2020,7 +2020,7 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -2063,7 +2063,7 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -2100,7 +2100,7 @@
         <v>15.96</v>
       </c>
       <c r="H34" t="n">
-        <v>15.9705</v>
+        <v>15.983</v>
       </c>
       <c r="I34" t="n">
         <v>55.08</v>
@@ -2112,7 +2112,7 @@
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -2161,7 +2161,7 @@
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -2210,7 +2210,7 @@
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -2244,7 +2244,7 @@
         </is>
       </c>
       <c r="G37" t="n">
-        <v>12.50300025939941</v>
+        <v>12.50399971008301</v>
       </c>
       <c r="J37" s="1" t="inlineStr">
         <is>
@@ -2253,7 +2253,7 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -2302,7 +2302,7 @@
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -2351,7 +2351,7 @@
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -2385,7 +2385,7 @@
         </is>
       </c>
       <c r="G40" t="n">
-        <v>113.1480026245117</v>
+        <v>113.1679992675781</v>
       </c>
       <c r="H40" t="n">
         <v>113.0768</v>
@@ -2400,7 +2400,7 @@
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -2449,7 +2449,7 @@
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -2498,7 +2498,7 @@
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -2547,7 +2547,7 @@
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -2584,19 +2584,19 @@
         <v>106.12</v>
       </c>
       <c r="H44" t="n">
-        <v>106.096</v>
+        <v>106.106</v>
       </c>
       <c r="I44" t="n">
         <v>100</v>
       </c>
-      <c r="J44" s="1" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+      <c r="J44" s="3" t="inlineStr">
+        <is>
+          <t>SELL</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -2645,7 +2645,7 @@
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -2694,7 +2694,7 @@
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -2743,7 +2743,7 @@
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -2792,7 +2792,7 @@
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -2841,7 +2841,7 @@
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -2890,7 +2890,7 @@
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -2939,7 +2939,7 @@
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -2988,7 +2988,7 @@
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -3037,7 +3037,7 @@
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -3086,7 +3086,7 @@
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -3135,7 +3135,7 @@
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -3184,7 +3184,7 @@
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -3233,7 +3233,7 @@
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -3282,7 +3282,7 @@
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -3331,7 +3331,7 @@
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -3380,7 +3380,7 @@
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -3429,7 +3429,7 @@
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -3478,7 +3478,7 @@
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -3512,7 +3512,7 @@
         </is>
       </c>
       <c r="G63" t="n">
-        <v>81.03</v>
+        <v>81.02999877929688</v>
       </c>
       <c r="H63" t="n">
         <v>77.80200000000001</v>
@@ -3520,14 +3520,14 @@
       <c r="I63" t="n">
         <v>63.81</v>
       </c>
-      <c r="J63" s="2" t="inlineStr">
-        <is>
-          <t>BUY</t>
+      <c r="J63" s="1" t="inlineStr">
+        <is>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -3576,7 +3576,7 @@
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -3625,7 +3625,7 @@
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -3674,7 +3674,7 @@
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -3723,7 +3723,7 @@
       </c>
       <c r="K67" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -3772,7 +3772,7 @@
       </c>
       <c r="K68" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -3821,7 +3821,7 @@
       </c>
       <c r="K69" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       </c>
       <c r="K70" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -3919,7 +3919,7 @@
       </c>
       <c r="K71" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -3968,7 +3968,7 @@
       </c>
       <c r="K72" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -4011,7 +4011,7 @@
       </c>
       <c r="K73" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -4048,7 +4048,7 @@
         <v>346.35</v>
       </c>
       <c r="H74" t="n">
-        <v>348.8645</v>
+        <v>347.948</v>
       </c>
       <c r="I74" t="n">
         <v>31.33</v>
@@ -4060,7 +4060,7 @@
       </c>
       <c r="K74" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -4094,7 +4094,7 @@
         </is>
       </c>
       <c r="G75" t="n">
-        <v>2658.722900390625</v>
+        <v>2658.577880859375</v>
       </c>
       <c r="J75" s="1" t="inlineStr">
         <is>
@@ -4103,7 +4103,7 @@
       </c>
       <c r="K75" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -4140,7 +4140,7 @@
         <v>280.03</v>
       </c>
       <c r="H76" t="n">
-        <v>278.533</v>
+        <v>278.456</v>
       </c>
       <c r="I76" t="n">
         <v>47.96</v>
@@ -4152,7 +4152,7 @@
       </c>
       <c r="K76" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -4201,7 +4201,7 @@
       </c>
       <c r="K77" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -4244,7 +4244,7 @@
       </c>
       <c r="K78" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -4287,7 +4287,7 @@
       </c>
       <c r="K79" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -4321,7 +4321,7 @@
         </is>
       </c>
       <c r="G80" t="n">
-        <v>212.9100036621094</v>
+        <v>213.4109954833984</v>
       </c>
       <c r="J80" s="1" t="inlineStr">
         <is>
@@ -4330,12 +4330,12 @@
       </c>
       <c r="K80" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
     <row r="81">
-      <c r="A81" t="n">
+      <c r="A81" s="4" t="n">
         <v>2</v>
       </c>
       <c r="B81" t="inlineStr">
@@ -4367,7 +4367,7 @@
         <v>190.82</v>
       </c>
       <c r="H81" t="n">
-        <v>189.5985</v>
+        <v>189.8105</v>
       </c>
       <c r="I81" t="n">
         <v>62.27</v>
@@ -4379,7 +4379,7 @@
       </c>
       <c r="K81" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -4416,7 +4416,7 @@
         <v>68.81999999999999</v>
       </c>
       <c r="H82" t="n">
-        <v>69.0185</v>
+        <v>68.9495</v>
       </c>
       <c r="I82" t="n">
         <v>35.68</v>
@@ -4428,7 +4428,7 @@
       </c>
       <c r="K82" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -4471,7 +4471,7 @@
       </c>
       <c r="K83" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -4508,7 +4508,7 @@
         <v>72.61</v>
       </c>
       <c r="H84" t="n">
-        <v>72.8115</v>
+        <v>72.7415</v>
       </c>
       <c r="I84" t="n">
         <v>36.35</v>
@@ -4520,7 +4520,7 @@
       </c>
       <c r="K84" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -4563,7 +4563,7 @@
       </c>
       <c r="K85" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -4600,7 +4600,7 @@
         <v>191.32</v>
       </c>
       <c r="H86" t="n">
-        <v>191.6595</v>
+        <v>191.6035</v>
       </c>
       <c r="I86" t="n">
         <v>39.1</v>
@@ -4612,7 +4612,7 @@
       </c>
       <c r="K86" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -4655,7 +4655,7 @@
       </c>
       <c r="K87" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -4698,7 +4698,7 @@
       </c>
       <c r="K88" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
@@ -4735,7 +4735,7 @@
         <v>976.27</v>
       </c>
       <c r="H89" t="n">
-        <v>979.1155</v>
+        <v>978.0105</v>
       </c>
       <c r="I89" t="n">
         <v>32.23</v>
@@ -4747,12 +4747,12 @@
       </c>
       <c r="K89" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>
     <row r="90">
-      <c r="A90" t="n">
+      <c r="A90" s="4" t="n">
         <v>2</v>
       </c>
       <c r="B90" t="inlineStr">
@@ -4784,7 +4784,7 @@
         <v>178.94</v>
       </c>
       <c r="H90" t="n">
-        <v>177.819</v>
+        <v>178.009</v>
       </c>
       <c r="I90" t="n">
         <v>61.96</v>
@@ -4796,7 +4796,7 @@
       </c>
       <c r="K90" t="inlineStr">
         <is>
-          <t>2026-02-24 15:05</t>
+          <t>2026-02-24 16:02</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix: rimuovi Carmignac Credit LU1623762843 da watchlist (hang FT Markets)
Il fondo causa hang indefinito nel fetch dati da FT Markets.
Spostato in Fondi_Rimossi per non bloccare il monitor run giornaliero.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fondi_monitoraggio.xlsx
+++ b/fondi_monitoraggio.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K90"/>
+  <dimension ref="A1:K89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -535,22 +535,22 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>291.67</v>
+        <v>296.91</v>
       </c>
       <c r="H2" t="n">
-        <v>288.1415</v>
+        <v>289.2315</v>
       </c>
       <c r="I2" t="n">
-        <v>61.92</v>
-      </c>
-      <c r="J2" s="1" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+        <v>71.08</v>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -584,13 +584,13 @@
         </is>
       </c>
       <c r="G3" t="n">
-        <v>369.06</v>
+        <v>380.52</v>
       </c>
       <c r="H3" t="n">
-        <v>352.627</v>
+        <v>355.4335</v>
       </c>
       <c r="I3" t="n">
-        <v>63.63</v>
+        <v>69.92</v>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
@@ -599,7 +599,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -633,13 +633,13 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>315.41</v>
+        <v>325.2</v>
       </c>
       <c r="H4" t="n">
-        <v>301.397</v>
+        <v>303.791</v>
       </c>
       <c r="I4" t="n">
-        <v>65.02</v>
+        <v>70.58</v>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
@@ -648,7 +648,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -682,13 +682,13 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>18.95</v>
+        <v>19.23</v>
       </c>
       <c r="H5" t="n">
-        <v>18.4835</v>
+        <v>18.563</v>
       </c>
       <c r="I5" t="n">
-        <v>65.36</v>
+        <v>70.08</v>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
@@ -697,7 +697,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -731,13 +731,13 @@
         </is>
       </c>
       <c r="G6" t="n">
-        <v>19.99</v>
+        <v>20.04</v>
       </c>
       <c r="H6" t="n">
-        <v>20.0685</v>
+        <v>20.0695</v>
       </c>
       <c r="I6" t="n">
-        <v>42.22</v>
+        <v>49.53</v>
       </c>
       <c r="J6" s="1" t="inlineStr">
         <is>
@@ -746,7 +746,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -780,7 +780,7 @@
         </is>
       </c>
       <c r="G7" t="n">
-        <v>51.1</v>
+        <v>51.08</v>
       </c>
       <c r="H7" t="n">
         <v>51.951</v>
@@ -795,7 +795,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -829,13 +829,13 @@
         </is>
       </c>
       <c r="G8" t="n">
-        <v>125.74</v>
+        <v>125.72</v>
       </c>
       <c r="H8" t="n">
-        <v>125.6295</v>
+        <v>125.6435</v>
       </c>
       <c r="I8" t="n">
-        <v>79.52</v>
+        <v>74.39</v>
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
@@ -844,7 +844,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -878,13 +878,13 @@
         </is>
       </c>
       <c r="G9" t="n">
-        <v>94.98</v>
+        <v>94.97</v>
       </c>
       <c r="H9" t="n">
-        <v>94.8905</v>
+        <v>94.9025</v>
       </c>
       <c r="I9" t="n">
-        <v>82.16</v>
+        <v>78.56</v>
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
@@ -893,7 +893,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -927,13 +927,13 @@
         </is>
       </c>
       <c r="G10" t="n">
-        <v>17.13</v>
+        <v>17.14</v>
       </c>
       <c r="H10" t="n">
-        <v>17.1255</v>
+        <v>17.1275</v>
       </c>
       <c r="I10" t="n">
-        <v>69.59999999999999</v>
+        <v>76.48999999999999</v>
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
@@ -942,7 +942,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -979,7 +979,7 @@
         <v>7.68</v>
       </c>
       <c r="H11" t="n">
-        <v>7.6745</v>
+        <v>7.6755</v>
       </c>
       <c r="I11" t="n">
         <v>68.19</v>
@@ -991,7 +991,7 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -1028,7 +1028,7 @@
         <v>10.83</v>
       </c>
       <c r="H12" t="n">
-        <v>10.825</v>
+        <v>10.826</v>
       </c>
       <c r="I12" t="n">
         <v>74.66</v>
@@ -1040,7 +1040,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -1074,13 +1074,13 @@
         </is>
       </c>
       <c r="G13" t="n">
-        <v>123.08</v>
+        <v>123.11</v>
       </c>
       <c r="H13" t="n">
-        <v>122.9215</v>
+        <v>122.947</v>
       </c>
       <c r="I13" t="n">
-        <v>62.65</v>
+        <v>64.3</v>
       </c>
       <c r="J13" s="1" t="inlineStr">
         <is>
@@ -1089,7 +1089,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -1123,13 +1123,13 @@
         </is>
       </c>
       <c r="G14" t="n">
-        <v>149.61</v>
+        <v>149.73</v>
       </c>
       <c r="H14" t="n">
-        <v>149.544</v>
+        <v>149.561</v>
       </c>
       <c r="I14" t="n">
-        <v>54.78</v>
+        <v>62.47</v>
       </c>
       <c r="J14" s="1" t="inlineStr">
         <is>
@@ -1138,7 +1138,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -1172,13 +1172,13 @@
         </is>
       </c>
       <c r="G15" t="n">
-        <v>56.76</v>
+        <v>58.06</v>
       </c>
       <c r="H15" t="n">
-        <v>57.3735</v>
+        <v>57.393</v>
       </c>
       <c r="I15" t="n">
-        <v>37.35</v>
+        <v>55.14</v>
       </c>
       <c r="J15" s="1" t="inlineStr">
         <is>
@@ -1187,7 +1187,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -1221,13 +1221,13 @@
         </is>
       </c>
       <c r="G16" t="n">
-        <v>22.51</v>
+        <v>22.53</v>
       </c>
       <c r="H16" t="n">
-        <v>22.367</v>
+        <v>22.387</v>
       </c>
       <c r="I16" t="n">
-        <v>52.57</v>
+        <v>52.97</v>
       </c>
       <c r="J16" s="1" t="inlineStr">
         <is>
@@ -1236,7 +1236,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -1270,7 +1270,7 @@
         </is>
       </c>
       <c r="G17" t="n">
-        <v>18.27</v>
+        <v>18.78</v>
       </c>
       <c r="H17" t="n">
         <v>18.1005</v>
@@ -1285,7 +1285,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -1319,13 +1319,13 @@
         </is>
       </c>
       <c r="G18" t="n">
-        <v>71.75</v>
+        <v>73.39</v>
       </c>
       <c r="H18" t="n">
-        <v>72.5335</v>
+        <v>72.5565</v>
       </c>
       <c r="I18" t="n">
-        <v>37.19</v>
+        <v>55</v>
       </c>
       <c r="J18" s="1" t="inlineStr">
         <is>
@@ -1334,7 +1334,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -1368,22 +1368,22 @@
         </is>
       </c>
       <c r="G19" t="n">
-        <v>15.17</v>
+        <v>15.57</v>
       </c>
       <c r="H19" t="n">
-        <v>15.031</v>
+        <v>15.0735</v>
       </c>
       <c r="I19" t="n">
-        <v>63.25</v>
-      </c>
-      <c r="J19" s="1" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+        <v>72.56999999999999</v>
+      </c>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>SELL</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -1417,13 +1417,13 @@
         </is>
       </c>
       <c r="G20" t="n">
-        <v>20.1</v>
+        <v>20.19</v>
       </c>
       <c r="H20" t="n">
-        <v>19.8125</v>
+        <v>19.8565</v>
       </c>
       <c r="I20" t="n">
-        <v>67.68000000000001</v>
+        <v>69.73999999999999</v>
       </c>
       <c r="J20" s="1" t="inlineStr">
         <is>
@@ -1432,7 +1432,7 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -1466,13 +1466,13 @@
         </is>
       </c>
       <c r="G21" t="n">
-        <v>116.14</v>
+        <v>115.37</v>
       </c>
       <c r="H21" t="n">
-        <v>114.377</v>
+        <v>114.5695</v>
       </c>
       <c r="I21" t="n">
-        <v>67.59</v>
+        <v>61.47</v>
       </c>
       <c r="J21" s="1" t="inlineStr">
         <is>
@@ -1481,7 +1481,7 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -1515,7 +1515,7 @@
         </is>
       </c>
       <c r="G22" t="n">
-        <v>8.220000000000001</v>
+        <v>8.48</v>
       </c>
       <c r="H22" t="n">
         <v>7.9335</v>
@@ -1530,7 +1530,7 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -1564,13 +1564,13 @@
         </is>
       </c>
       <c r="G23" t="n">
-        <v>32.65</v>
+        <v>32.71</v>
       </c>
       <c r="H23" t="n">
-        <v>32.583</v>
+        <v>32.5935</v>
       </c>
       <c r="I23" t="n">
-        <v>56.51</v>
+        <v>57.83</v>
       </c>
       <c r="J23" s="1" t="inlineStr">
         <is>
@@ -1579,7 +1579,7 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -1613,7 +1613,7 @@
         </is>
       </c>
       <c r="G24" t="n">
-        <v>7.65</v>
+        <v>7.57</v>
       </c>
       <c r="H24" t="n">
         <v>7.2805</v>
@@ -1628,7 +1628,7 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -1662,13 +1662,13 @@
         </is>
       </c>
       <c r="G25" t="n">
-        <v>1382.77</v>
+        <v>1410.59</v>
       </c>
       <c r="H25" t="n">
-        <v>1345.8625</v>
+        <v>1350.6905</v>
       </c>
       <c r="I25" t="n">
-        <v>68.48</v>
+        <v>73.91</v>
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
@@ -1677,7 +1677,7 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -1711,7 +1711,7 @@
         </is>
       </c>
       <c r="G26" t="n">
-        <v>101.12</v>
+        <v>101.24</v>
       </c>
       <c r="H26" t="n">
         <v>33.9061</v>
@@ -1726,7 +1726,7 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -1760,13 +1760,13 @@
         </is>
       </c>
       <c r="G27" t="n">
-        <v>19.18</v>
+        <v>19.32</v>
       </c>
       <c r="H27" t="n">
-        <v>18.942</v>
+        <v>18.9775</v>
       </c>
       <c r="I27" t="n">
-        <v>66</v>
+        <v>70.31</v>
       </c>
       <c r="J27" s="1" t="inlineStr">
         <is>
@@ -1775,7 +1775,7 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -1809,22 +1809,22 @@
         </is>
       </c>
       <c r="G28" t="n">
-        <v>21.94</v>
+        <v>22.65</v>
       </c>
       <c r="H28" t="n">
-        <v>21.6945</v>
+        <v>21.7815</v>
       </c>
       <c r="I28" t="n">
-        <v>68.38</v>
-      </c>
-      <c r="J28" s="1" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+        <v>81.16</v>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -1858,13 +1858,13 @@
         </is>
       </c>
       <c r="G29" t="n">
-        <v>62.45</v>
+        <v>62.66</v>
       </c>
       <c r="H29" t="n">
-        <v>62.2185</v>
+        <v>62.26</v>
       </c>
       <c r="I29" t="n">
-        <v>50.07</v>
+        <v>55.28</v>
       </c>
       <c r="J29" s="1" t="inlineStr">
         <is>
@@ -1873,7 +1873,7 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -1907,7 +1907,7 @@
         </is>
       </c>
       <c r="G30" t="n">
-        <v>282.1</v>
+        <v>283.65</v>
       </c>
       <c r="H30" t="n">
         <v>281.0385</v>
@@ -1922,7 +1922,7 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -1956,7 +1956,7 @@
         </is>
       </c>
       <c r="G31" t="n">
-        <v>25.03</v>
+        <v>25.14</v>
       </c>
       <c r="H31" t="n">
         <v>25.655</v>
@@ -1971,7 +1971,7 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -2005,7 +2005,7 @@
         </is>
       </c>
       <c r="G32" t="n">
-        <v>32.43000030517578</v>
+        <v>32.61999893188477</v>
       </c>
       <c r="H32" t="n">
         <v>31.8945</v>
@@ -2020,7 +2020,7 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -2054,7 +2054,7 @@
         </is>
       </c>
       <c r="G33" t="n">
-        <v>72.25199890136719</v>
+        <v>72.44599914550781</v>
       </c>
       <c r="J33" s="1" t="inlineStr">
         <is>
@@ -2063,7 +2063,7 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -2097,13 +2097,13 @@
         </is>
       </c>
       <c r="G34" t="n">
-        <v>15.96</v>
+        <v>16.07</v>
       </c>
       <c r="H34" t="n">
-        <v>15.983</v>
+        <v>15.9835</v>
       </c>
       <c r="I34" t="n">
-        <v>55.08</v>
+        <v>62.64</v>
       </c>
       <c r="J34" s="1" t="inlineStr">
         <is>
@@ -2112,7 +2112,7 @@
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -2146,7 +2146,7 @@
         </is>
       </c>
       <c r="G35" t="n">
-        <v>203.06</v>
+        <v>204.84</v>
       </c>
       <c r="H35" t="n">
         <v>200.7005</v>
@@ -2161,7 +2161,7 @@
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -2195,7 +2195,7 @@
         </is>
       </c>
       <c r="G36" t="n">
-        <v>31.76</v>
+        <v>32.25</v>
       </c>
       <c r="H36" t="n">
         <v>31.87</v>
@@ -2210,7 +2210,7 @@
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -2244,7 +2244,7 @@
         </is>
       </c>
       <c r="G37" t="n">
-        <v>12.50399971008301</v>
+        <v>12.55599975585938</v>
       </c>
       <c r="J37" s="1" t="inlineStr">
         <is>
@@ -2253,7 +2253,7 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -2287,7 +2287,7 @@
         </is>
       </c>
       <c r="G38" t="n">
-        <v>243.94</v>
+        <v>246.09</v>
       </c>
       <c r="H38" t="n">
         <v>240.2335</v>
@@ -2302,7 +2302,7 @@
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -2336,7 +2336,7 @@
         </is>
       </c>
       <c r="G39" t="n">
-        <v>157.01</v>
+        <v>157.03</v>
       </c>
       <c r="H39" t="n">
         <v>157.212</v>
@@ -2351,7 +2351,7 @@
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -2385,7 +2385,7 @@
         </is>
       </c>
       <c r="G40" t="n">
-        <v>113.1679992675781</v>
+        <v>113.161003112793</v>
       </c>
       <c r="H40" t="n">
         <v>113.0768</v>
@@ -2400,7 +2400,7 @@
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -2434,7 +2434,7 @@
         </is>
       </c>
       <c r="G41" t="n">
-        <v>128.8000030517578</v>
+        <v>128.8600006103516</v>
       </c>
       <c r="H41" t="n">
         <v>128.617</v>
@@ -2449,7 +2449,7 @@
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -2483,7 +2483,7 @@
         </is>
       </c>
       <c r="G42" t="n">
-        <v>103.64</v>
+        <v>103.65</v>
       </c>
       <c r="H42" t="n">
         <v>103.392</v>
@@ -2498,7 +2498,7 @@
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -2532,7 +2532,7 @@
         </is>
       </c>
       <c r="G43" t="n">
-        <v>226.77</v>
+        <v>232.15</v>
       </c>
       <c r="H43" t="n">
         <v>219.028</v>
@@ -2547,7 +2547,7 @@
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -2581,22 +2581,22 @@
         </is>
       </c>
       <c r="G44" t="n">
-        <v>106.12</v>
+        <v>106.15</v>
       </c>
       <c r="H44" t="n">
-        <v>106.106</v>
+        <v>106.1105</v>
       </c>
       <c r="I44" t="n">
         <v>100</v>
       </c>
-      <c r="J44" s="3" t="inlineStr">
-        <is>
-          <t>SELL</t>
+      <c r="J44" s="1" t="inlineStr">
+        <is>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -2630,7 +2630,7 @@
         </is>
       </c>
       <c r="G45" t="n">
-        <v>82.33</v>
+        <v>84.08</v>
       </c>
       <c r="H45" t="n">
         <v>79.8175</v>
@@ -2645,7 +2645,7 @@
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -2679,7 +2679,7 @@
         </is>
       </c>
       <c r="G46" t="n">
-        <v>329.46</v>
+        <v>329.51</v>
       </c>
       <c r="H46" t="n">
         <v>316.654</v>
@@ -2694,7 +2694,7 @@
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -2728,7 +2728,7 @@
         </is>
       </c>
       <c r="G47" t="n">
-        <v>134.57</v>
+        <v>134.6</v>
       </c>
       <c r="H47" t="n">
         <v>133.8405</v>
@@ -2743,7 +2743,7 @@
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -2792,7 +2792,7 @@
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -2826,7 +2826,7 @@
         </is>
       </c>
       <c r="G49" t="n">
-        <v>111.9700012207031</v>
+        <v>111.4599990844727</v>
       </c>
       <c r="H49" t="n">
         <v>109.2185</v>
@@ -2841,7 +2841,7 @@
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -2875,7 +2875,7 @@
         </is>
       </c>
       <c r="G50" t="n">
-        <v>258.26</v>
+        <v>260.57</v>
       </c>
       <c r="H50" t="n">
         <v>256.88</v>
@@ -2890,7 +2890,7 @@
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -2924,7 +2924,7 @@
         </is>
       </c>
       <c r="G51" t="n">
-        <v>56.29000091552734</v>
+        <v>56.06000137329102</v>
       </c>
       <c r="H51" t="n">
         <v>55.1783</v>
@@ -2939,7 +2939,7 @@
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -2973,7 +2973,7 @@
         </is>
       </c>
       <c r="G52" t="n">
-        <v>221.39</v>
+        <v>222.52</v>
       </c>
       <c r="H52" t="n">
         <v>221.319</v>
@@ -2988,7 +2988,7 @@
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -3022,7 +3022,7 @@
         </is>
       </c>
       <c r="G53" t="n">
-        <v>50.42</v>
+        <v>50.47</v>
       </c>
       <c r="H53" t="n">
         <v>50.3505</v>
@@ -3037,7 +3037,7 @@
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -3071,7 +3071,7 @@
         </is>
       </c>
       <c r="G54" t="n">
-        <v>46.97</v>
+        <v>46.93</v>
       </c>
       <c r="H54" t="n">
         <v>46.734</v>
@@ -3086,7 +3086,7 @@
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -3120,7 +3120,7 @@
         </is>
       </c>
       <c r="G55" t="n">
-        <v>88.23999786376953</v>
+        <v>87.55000305175781</v>
       </c>
       <c r="H55" t="n">
         <v>87.523</v>
@@ -3135,7 +3135,7 @@
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -3169,7 +3169,7 @@
         </is>
       </c>
       <c r="G56" t="n">
-        <v>488.1400146484375</v>
+        <v>484.4700012207031</v>
       </c>
       <c r="H56" t="n">
         <v>477.475</v>
@@ -3184,7 +3184,7 @@
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -3218,7 +3218,7 @@
         </is>
       </c>
       <c r="G57" t="n">
-        <v>114.07</v>
+        <v>114.15</v>
       </c>
       <c r="H57" t="n">
         <v>113.925</v>
@@ -3233,7 +3233,7 @@
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -3267,7 +3267,7 @@
         </is>
       </c>
       <c r="G58" t="n">
-        <v>105.32</v>
+        <v>105.21</v>
       </c>
       <c r="H58" t="n">
         <v>105.189</v>
@@ -3282,7 +3282,7 @@
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -3316,7 +3316,7 @@
         </is>
       </c>
       <c r="G59" t="n">
-        <v>170.5</v>
+        <v>170.6600036621094</v>
       </c>
       <c r="H59" t="n">
         <v>169.8945</v>
@@ -3331,7 +3331,7 @@
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="G60" t="n">
-        <v>75.29000000000001</v>
+        <v>75.26000000000001</v>
       </c>
       <c r="H60" t="n">
         <v>75.00149999999999</v>
@@ -3380,7 +3380,7 @@
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -3414,7 +3414,7 @@
         </is>
       </c>
       <c r="G61" t="n">
-        <v>106.05</v>
+        <v>105.99</v>
       </c>
       <c r="H61" t="n">
         <v>105.9255</v>
@@ -3429,7 +3429,7 @@
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -3463,7 +3463,7 @@
         </is>
       </c>
       <c r="G62" t="n">
-        <v>56.68999862670898</v>
+        <v>56.40999984741211</v>
       </c>
       <c r="H62" t="n">
         <v>56.2893</v>
@@ -3478,7 +3478,7 @@
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -3512,7 +3512,7 @@
         </is>
       </c>
       <c r="G63" t="n">
-        <v>81.02999877929688</v>
+        <v>80.62000274658203</v>
       </c>
       <c r="H63" t="n">
         <v>77.80200000000001</v>
@@ -3527,7 +3527,7 @@
       </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -3561,7 +3561,7 @@
         </is>
       </c>
       <c r="G64" t="n">
-        <v>126.36</v>
+        <v>128.36</v>
       </c>
       <c r="H64" t="n">
         <v>123.431</v>
@@ -3576,7 +3576,7 @@
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -3610,7 +3610,7 @@
         </is>
       </c>
       <c r="G65" t="n">
-        <v>118.04</v>
+        <v>118.01</v>
       </c>
       <c r="H65" t="n">
         <v>117.8</v>
@@ -3625,7 +3625,7 @@
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -3674,7 +3674,7 @@
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -3708,7 +3708,7 @@
         </is>
       </c>
       <c r="G67" t="n">
-        <v>53.09</v>
+        <v>53.03</v>
       </c>
       <c r="H67" t="n">
         <v>52.463</v>
@@ -3723,7 +3723,7 @@
       </c>
       <c r="K67" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -3757,7 +3757,7 @@
         </is>
       </c>
       <c r="G68" t="n">
-        <v>58.06000137329102</v>
+        <v>58.06999969482422</v>
       </c>
       <c r="H68" t="n">
         <v>57.7105</v>
@@ -3772,7 +3772,7 @@
       </c>
       <c r="K68" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -3806,7 +3806,7 @@
         </is>
       </c>
       <c r="G69" t="n">
-        <v>50.64</v>
+        <v>50.6</v>
       </c>
       <c r="H69" t="n">
         <v>50.331</v>
@@ -3821,7 +3821,7 @@
       </c>
       <c r="K69" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -3855,7 +3855,7 @@
         </is>
       </c>
       <c r="G70" t="n">
-        <v>550.7</v>
+        <v>562.75</v>
       </c>
       <c r="H70" t="n">
         <v>567.1135</v>
@@ -3870,7 +3870,7 @@
       </c>
       <c r="K70" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -3904,7 +3904,7 @@
         </is>
       </c>
       <c r="G71" t="n">
-        <v>24.16</v>
+        <v>24.59</v>
       </c>
       <c r="H71" t="n">
         <v>23.984</v>
@@ -3919,7 +3919,7 @@
       </c>
       <c r="K71" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -3953,7 +3953,7 @@
         </is>
       </c>
       <c r="G72" t="n">
-        <v>80.56999999999999</v>
+        <v>81.53</v>
       </c>
       <c r="H72" t="n">
         <v>81.0485</v>
@@ -3968,7 +3968,7 @@
       </c>
       <c r="K72" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -4002,7 +4002,7 @@
         </is>
       </c>
       <c r="G73" t="n">
-        <v>1926.119995117188</v>
+        <v>1926.787963867188</v>
       </c>
       <c r="J73" s="1" t="inlineStr">
         <is>
@@ -4011,7 +4011,7 @@
       </c>
       <c r="K73" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -4045,13 +4045,13 @@
         </is>
       </c>
       <c r="G74" t="n">
-        <v>346.35</v>
+        <v>355.64</v>
       </c>
       <c r="H74" t="n">
-        <v>347.948</v>
+        <v>348.33</v>
       </c>
       <c r="I74" t="n">
-        <v>31.33</v>
+        <v>61.47</v>
       </c>
       <c r="J74" s="1" t="inlineStr">
         <is>
@@ -4060,7 +4060,7 @@
       </c>
       <c r="K74" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -4094,7 +4094,7 @@
         </is>
       </c>
       <c r="G75" t="n">
-        <v>2658.577880859375</v>
+        <v>2717.27099609375</v>
       </c>
       <c r="J75" s="1" t="inlineStr">
         <is>
@@ -4103,7 +4103,7 @@
       </c>
       <c r="K75" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -4137,13 +4137,13 @@
         </is>
       </c>
       <c r="G76" t="n">
-        <v>280.03</v>
+        <v>279.91</v>
       </c>
       <c r="H76" t="n">
-        <v>278.456</v>
+        <v>278.601</v>
       </c>
       <c r="I76" t="n">
-        <v>47.96</v>
+        <v>47.36</v>
       </c>
       <c r="J76" s="1" t="inlineStr">
         <is>
@@ -4152,22 +4152,22 @@
       </c>
       <c r="K76" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>LU1623762843</t>
+          <t>FR0010149302</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Carmignac Credit A EUR Acc</t>
+          <t>Carmignac Emergents A EUR Acc</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -4186,13 +4186,7 @@
         </is>
       </c>
       <c r="G77" t="n">
-        <v>159.9700012207031</v>
-      </c>
-      <c r="H77" t="n">
-        <v>159.493</v>
-      </c>
-      <c r="I77" t="n">
-        <v>77.12</v>
+        <v>1650.0419921875</v>
       </c>
       <c r="J77" s="1" t="inlineStr">
         <is>
@@ -4201,7 +4195,7 @@
       </c>
       <c r="K77" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -4211,12 +4205,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>FR0010149302</t>
+          <t>FR0011269083</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Carmignac Emergents A EUR Acc</t>
+          <t>Carmignac Sécurité AW EUR Ydis</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -4226,7 +4220,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Altri</t>
+          <t>Fondi Flessibili</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -4235,7 +4229,7 @@
         </is>
       </c>
       <c r="G78" t="n">
-        <v>1638.321044921875</v>
+        <v>99.56800079345703</v>
       </c>
       <c r="J78" s="1" t="inlineStr">
         <is>
@@ -4244,7 +4238,7 @@
       </c>
       <c r="K78" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -4254,12 +4248,12 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>FR0011269083</t>
+          <t>FR0011269349</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Carmignac Sécurité AW EUR Ydis</t>
+          <t>Carmignac Emergents A EUR Ydis</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -4269,7 +4263,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Fondi Flessibili</t>
+          <t>Azionari Paesi Emergenti</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -4278,7 +4272,7 @@
         </is>
       </c>
       <c r="G79" t="n">
-        <v>99.56800079345703</v>
+        <v>215.6589965820312</v>
       </c>
       <c r="J79" s="1" t="inlineStr">
         <is>
@@ -4287,22 +4281,22 @@
       </c>
       <c r="K79" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
     <row r="80">
-      <c r="A80" t="n">
-        <v>3</v>
+      <c r="A80" s="4" t="n">
+        <v>2</v>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>FR0011269349</t>
+          <t>LU1317704051</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Carmignac Emergents A EUR Ydis</t>
+          <t>Carmignac Long-Short Europ. Eqs A EUR Acc</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -4312,7 +4306,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Azionari Paesi Emergenti</t>
+          <t>Altri</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -4321,7 +4315,13 @@
         </is>
       </c>
       <c r="G80" t="n">
-        <v>213.4109954833984</v>
+        <v>190.63</v>
+      </c>
+      <c r="H80" t="n">
+        <v>189.8945</v>
+      </c>
+      <c r="I80" t="n">
+        <v>59.29</v>
       </c>
       <c r="J80" s="1" t="inlineStr">
         <is>
@@ -4330,22 +4330,22 @@
       </c>
       <c r="K80" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="4" t="n">
-        <v>2</v>
+      <c r="A81" t="n">
+        <v>3</v>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>LU1317704051</t>
+          <t>LU1163533349</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Carmignac Long-Short Europ. Eqs A EUR Acc</t>
+          <t>Carmignac Patrimoine E EUR Minc</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -4364,13 +4364,13 @@
         </is>
       </c>
       <c r="G81" t="n">
-        <v>190.82</v>
+        <v>69.37</v>
       </c>
       <c r="H81" t="n">
-        <v>189.8105</v>
+        <v>68.967</v>
       </c>
       <c r="I81" t="n">
-        <v>62.27</v>
+        <v>54.11</v>
       </c>
       <c r="J81" s="1" t="inlineStr">
         <is>
@@ -4379,7 +4379,7 @@
       </c>
       <c r="K81" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -4389,12 +4389,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>LU1163533349</t>
+          <t>FR0011269588</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Carmignac Patrimoine E EUR Minc</t>
+          <t>Carmignac Patrimoine A EUR Ydis</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -4404,7 +4404,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Altri</t>
+          <t>Bilanciati</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -4413,13 +4413,7 @@
         </is>
       </c>
       <c r="G82" t="n">
-        <v>68.81999999999999</v>
-      </c>
-      <c r="H82" t="n">
-        <v>68.9495</v>
-      </c>
-      <c r="I82" t="n">
-        <v>35.68</v>
+        <v>128.2530059814453</v>
       </c>
       <c r="J82" s="1" t="inlineStr">
         <is>
@@ -4428,7 +4422,7 @@
       </c>
       <c r="K82" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -4438,12 +4432,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>FR0011269588</t>
+          <t>LU1163533422</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Carmignac Patrimoine A EUR Ydis</t>
+          <t>Carmignac Patrimoine A EUR Minc</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -4453,7 +4447,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Bilanciati</t>
+          <t>Altri</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -4462,7 +4456,13 @@
         </is>
       </c>
       <c r="G83" t="n">
-        <v>127.3740005493164</v>
+        <v>73.19</v>
+      </c>
+      <c r="H83" t="n">
+        <v>72.76049999999999</v>
+      </c>
+      <c r="I83" t="n">
+        <v>54.86</v>
       </c>
       <c r="J83" s="1" t="inlineStr">
         <is>
@@ -4471,7 +4471,7 @@
       </c>
       <c r="K83" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -4481,12 +4481,12 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>LU1163533422</t>
+          <t>FR0010135103</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Carmignac Patrimoine A EUR Minc</t>
+          <t>Carmignac Patrimoine A EUR Acc</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -4496,7 +4496,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Altri</t>
+          <t>Bilanciati</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -4505,13 +4505,7 @@
         </is>
       </c>
       <c r="G84" t="n">
-        <v>72.61</v>
-      </c>
-      <c r="H84" t="n">
-        <v>72.7415</v>
-      </c>
-      <c r="I84" t="n">
-        <v>36.35</v>
+        <v>800.5250244140625</v>
       </c>
       <c r="J84" s="1" t="inlineStr">
         <is>
@@ -4520,7 +4514,7 @@
       </c>
       <c r="K84" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -4530,12 +4524,12 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>FR0010135103</t>
+          <t>FR0010306142</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Carmignac Patrimoine A EUR Acc</t>
+          <t>Carmignac Patrimoine E EUR Acc</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -4554,7 +4548,13 @@
         </is>
       </c>
       <c r="G85" t="n">
-        <v>798.1339721679688</v>
+        <v>192.75</v>
+      </c>
+      <c r="H85" t="n">
+        <v>191.6865</v>
+      </c>
+      <c r="I85" t="n">
+        <v>57.09</v>
       </c>
       <c r="J85" s="1" t="inlineStr">
         <is>
@@ -4563,7 +4563,7 @@
       </c>
       <c r="K85" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -4573,12 +4573,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>FR0010306142</t>
+          <t>LU0336084032</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Carmignac Patrimoine E EUR Acc</t>
+          <t>Carmignac Flexible Bond A EUR Acc</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -4588,7 +4588,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Bilanciati</t>
+          <t>Obb. Misti</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -4597,13 +4597,7 @@
         </is>
       </c>
       <c r="G86" t="n">
-        <v>191.32</v>
-      </c>
-      <c r="H86" t="n">
-        <v>191.6035</v>
-      </c>
-      <c r="I86" t="n">
-        <v>39.1</v>
+        <v>1380.400024414062</v>
       </c>
       <c r="J86" s="1" t="inlineStr">
         <is>
@@ -4612,7 +4606,7 @@
       </c>
       <c r="K86" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -4622,12 +4616,12 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>LU0336084032</t>
+          <t>LU0992631050</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Carmignac Flexible Bond A EUR Acc</t>
+          <t>Carmignac Flexible Bond A EUR Ydis</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -4646,7 +4640,7 @@
         </is>
       </c>
       <c r="G87" t="n">
-        <v>1380.400024414062</v>
+        <v>1090.800048828125</v>
       </c>
       <c r="J87" s="1" t="inlineStr">
         <is>
@@ -4655,7 +4649,7 @@
       </c>
       <c r="K87" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -4665,12 +4659,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>LU0992631050</t>
+          <t>LU1299302684</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Carmignac Flexible Bond A EUR Ydis</t>
+          <t>Carmignac Flexible Bond A EUR Minc</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -4689,7 +4683,13 @@
         </is>
       </c>
       <c r="G88" t="n">
-        <v>1090.800048828125</v>
+        <v>976.88</v>
+      </c>
+      <c r="H88" t="n">
+        <v>977.7005</v>
+      </c>
+      <c r="I88" t="n">
+        <v>38.06</v>
       </c>
       <c r="J88" s="1" t="inlineStr">
         <is>
@@ -4698,22 +4698,22 @@
       </c>
       <c r="K88" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
     <row r="89">
-      <c r="A89" t="n">
-        <v>3</v>
+      <c r="A89" s="4" t="n">
+        <v>2</v>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>LU1299302684</t>
+          <t>LU1317704135</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Carmignac Flexible Bond A EUR Minc</t>
+          <t>Carmignac Long-Short Europ. Eqs E EUR Acc</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -4723,7 +4723,7 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Obb. Misti</t>
+          <t>Altri</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -4732,13 +4732,13 @@
         </is>
       </c>
       <c r="G89" t="n">
-        <v>976.27</v>
+        <v>178.75</v>
       </c>
       <c r="H89" t="n">
-        <v>978.0105</v>
+        <v>178.0845</v>
       </c>
       <c r="I89" t="n">
-        <v>32.23</v>
+        <v>58.8</v>
       </c>
       <c r="J89" s="1" t="inlineStr">
         <is>
@@ -4747,56 +4747,7 @@
       </c>
       <c r="K89" t="inlineStr">
         <is>
-          <t>2026-02-24 16:02</t>
-        </is>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="B90" t="inlineStr">
-        <is>
-          <t>LU1317704135</t>
-        </is>
-      </c>
-      <c r="C90" t="inlineStr">
-        <is>
-          <t>Carmignac Long-Short Europ. Eqs E EUR Acc</t>
-        </is>
-      </c>
-      <c r="D90" t="inlineStr">
-        <is>
-          <t>Carmignac</t>
-        </is>
-      </c>
-      <c r="E90" t="inlineStr">
-        <is>
-          <t>Altri</t>
-        </is>
-      </c>
-      <c r="F90" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="G90" t="n">
-        <v>178.94</v>
-      </c>
-      <c r="H90" t="n">
-        <v>178.009</v>
-      </c>
-      <c r="I90" t="n">
-        <v>61.96</v>
-      </c>
-      <c r="J90" s="1" t="inlineStr">
-        <is>
-          <t>HOLD</t>
-        </is>
-      </c>
-      <c r="K90" t="inlineStr">
-        <is>
-          <t>2026-02-24 16:02</t>
+          <t>2026-02-26 19:47</t>
         </is>
       </c>
     </row>
@@ -4811,7 +4762,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:M19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5115,6 +5066,65 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>2</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>LU1623762843</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Carmignac Credit A EUR Acc</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Carmignac</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Altri</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>160.0200042724609</v>
+      </c>
+      <c r="H19" t="n">
+        <v>159.493</v>
+      </c>
+      <c r="I19" t="n">
+        <v>77.12</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>2026-02-26 19:47</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>Hang su FT Markets</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix: rimuovi Carmignac Emergents A+Ydis da watchlist (hang FT Markets)
FR0010149302 - Carmignac Emergents A EUR Acc
FR0011269349 - Carmignac Emergents A EUR Ydis
Totale fondi watchlist: 86

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fondi_monitoraggio.xlsx
+++ b/fondi_monitoraggio.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K89"/>
+  <dimension ref="A1:K87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4162,12 +4162,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>FR0010149302</t>
+          <t>FR0011269083</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Carmignac Emergents A EUR Acc</t>
+          <t>Carmignac Sécurité AW EUR Ydis</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -4177,59 +4177,65 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
+          <t>Fondi Flessibili</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G77" t="n">
+        <v>99.56800079345703</v>
+      </c>
+      <c r="J77" s="1" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>2026-02-26 19:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>LU1317704051</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Carmignac Long-Short Europ. Eqs A EUR Acc</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Carmignac</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
           <t>Altri</t>
         </is>
       </c>
-      <c r="F77" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="G77" t="n">
-        <v>1650.0419921875</v>
-      </c>
-      <c r="J77" s="1" t="inlineStr">
-        <is>
-          <t>HOLD</t>
-        </is>
-      </c>
-      <c r="K77" t="inlineStr">
-        <is>
-          <t>2026-02-26 19:47</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" t="n">
-        <v>3</v>
-      </c>
-      <c r="B78" t="inlineStr">
-        <is>
-          <t>FR0011269083</t>
-        </is>
-      </c>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>Carmignac Sécurité AW EUR Ydis</t>
-        </is>
-      </c>
-      <c r="D78" t="inlineStr">
-        <is>
-          <t>Carmignac</t>
-        </is>
-      </c>
-      <c r="E78" t="inlineStr">
-        <is>
-          <t>Fondi Flessibili</t>
-        </is>
-      </c>
       <c r="F78" t="inlineStr">
         <is>
           <t>EUR</t>
         </is>
       </c>
       <c r="G78" t="n">
-        <v>99.56800079345703</v>
+        <v>190.63</v>
+      </c>
+      <c r="H78" t="n">
+        <v>189.8945</v>
+      </c>
+      <c r="I78" t="n">
+        <v>59.29</v>
       </c>
       <c r="J78" s="1" t="inlineStr">
         <is>
@@ -4248,12 +4254,12 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>FR0011269349</t>
+          <t>LU1163533349</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Carmignac Emergents A EUR Ydis</t>
+          <t>Carmignac Patrimoine E EUR Minc</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -4263,7 +4269,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Azionari Paesi Emergenti</t>
+          <t>Altri</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -4272,7 +4278,13 @@
         </is>
       </c>
       <c r="G79" t="n">
-        <v>215.6589965820312</v>
+        <v>69.37</v>
+      </c>
+      <c r="H79" t="n">
+        <v>68.967</v>
+      </c>
+      <c r="I79" t="n">
+        <v>54.11</v>
       </c>
       <c r="J79" s="1" t="inlineStr">
         <is>
@@ -4286,17 +4298,17 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="4" t="n">
-        <v>2</v>
+      <c r="A80" t="n">
+        <v>3</v>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>LU1317704051</t>
+          <t>FR0011269588</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Carmignac Long-Short Europ. Eqs A EUR Acc</t>
+          <t>Carmignac Patrimoine A EUR Ydis</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -4306,7 +4318,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Altri</t>
+          <t>Bilanciati</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -4315,13 +4327,7 @@
         </is>
       </c>
       <c r="G80" t="n">
-        <v>190.63</v>
-      </c>
-      <c r="H80" t="n">
-        <v>189.8945</v>
-      </c>
-      <c r="I80" t="n">
-        <v>59.29</v>
+        <v>128.2530059814453</v>
       </c>
       <c r="J80" s="1" t="inlineStr">
         <is>
@@ -4340,12 +4346,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>LU1163533349</t>
+          <t>LU1163533422</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Carmignac Patrimoine E EUR Minc</t>
+          <t>Carmignac Patrimoine A EUR Minc</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -4364,13 +4370,13 @@
         </is>
       </c>
       <c r="G81" t="n">
-        <v>69.37</v>
+        <v>73.19</v>
       </c>
       <c r="H81" t="n">
-        <v>68.967</v>
+        <v>72.76049999999999</v>
       </c>
       <c r="I81" t="n">
-        <v>54.11</v>
+        <v>54.86</v>
       </c>
       <c r="J81" s="1" t="inlineStr">
         <is>
@@ -4389,12 +4395,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>FR0011269588</t>
+          <t>FR0010135103</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Carmignac Patrimoine A EUR Ydis</t>
+          <t>Carmignac Patrimoine A EUR Acc</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -4413,7 +4419,7 @@
         </is>
       </c>
       <c r="G82" t="n">
-        <v>128.2530059814453</v>
+        <v>800.5250244140625</v>
       </c>
       <c r="J82" s="1" t="inlineStr">
         <is>
@@ -4432,12 +4438,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>LU1163533422</t>
+          <t>FR0010306142</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Carmignac Patrimoine A EUR Minc</t>
+          <t>Carmignac Patrimoine E EUR Acc</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -4447,7 +4453,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Altri</t>
+          <t>Bilanciati</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -4456,13 +4462,13 @@
         </is>
       </c>
       <c r="G83" t="n">
-        <v>73.19</v>
+        <v>192.75</v>
       </c>
       <c r="H83" t="n">
-        <v>72.76049999999999</v>
+        <v>191.6865</v>
       </c>
       <c r="I83" t="n">
-        <v>54.86</v>
+        <v>57.09</v>
       </c>
       <c r="J83" s="1" t="inlineStr">
         <is>
@@ -4481,12 +4487,12 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>FR0010135103</t>
+          <t>LU0336084032</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Carmignac Patrimoine A EUR Acc</t>
+          <t>Carmignac Flexible Bond A EUR Acc</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -4496,7 +4502,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Bilanciati</t>
+          <t>Obb. Misti</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -4505,7 +4511,7 @@
         </is>
       </c>
       <c r="G84" t="n">
-        <v>800.5250244140625</v>
+        <v>1380.400024414062</v>
       </c>
       <c r="J84" s="1" t="inlineStr">
         <is>
@@ -4524,12 +4530,12 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>FR0010306142</t>
+          <t>LU0992631050</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Carmignac Patrimoine E EUR Acc</t>
+          <t>Carmignac Flexible Bond A EUR Ydis</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -4539,7 +4545,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Bilanciati</t>
+          <t>Obb. Misti</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -4548,13 +4554,7 @@
         </is>
       </c>
       <c r="G85" t="n">
-        <v>192.75</v>
-      </c>
-      <c r="H85" t="n">
-        <v>191.6865</v>
-      </c>
-      <c r="I85" t="n">
-        <v>57.09</v>
+        <v>1090.800048828125</v>
       </c>
       <c r="J85" s="1" t="inlineStr">
         <is>
@@ -4573,12 +4573,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>LU0336084032</t>
+          <t>LU1299302684</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Carmignac Flexible Bond A EUR Acc</t>
+          <t>Carmignac Flexible Bond A EUR Minc</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -4597,7 +4597,13 @@
         </is>
       </c>
       <c r="G86" t="n">
-        <v>1380.400024414062</v>
+        <v>976.88</v>
+      </c>
+      <c r="H86" t="n">
+        <v>977.7005</v>
+      </c>
+      <c r="I86" t="n">
+        <v>38.06</v>
       </c>
       <c r="J86" s="1" t="inlineStr">
         <is>
@@ -4611,17 +4617,17 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" t="n">
-        <v>3</v>
+      <c r="A87" s="4" t="n">
+        <v>2</v>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>LU0992631050</t>
+          <t>LU1317704135</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Carmignac Flexible Bond A EUR Ydis</t>
+          <t>Carmignac Long-Short Europ. Eqs E EUR Acc</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -4631,7 +4637,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Obb. Misti</t>
+          <t>Altri</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -4640,7 +4646,13 @@
         </is>
       </c>
       <c r="G87" t="n">
-        <v>1090.800048828125</v>
+        <v>178.75</v>
+      </c>
+      <c r="H87" t="n">
+        <v>178.0845</v>
+      </c>
+      <c r="I87" t="n">
+        <v>58.8</v>
       </c>
       <c r="J87" s="1" t="inlineStr">
         <is>
@@ -4648,104 +4660,6 @@
         </is>
       </c>
       <c r="K87" t="inlineStr">
-        <is>
-          <t>2026-02-26 19:47</t>
-        </is>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" t="n">
-        <v>3</v>
-      </c>
-      <c r="B88" t="inlineStr">
-        <is>
-          <t>LU1299302684</t>
-        </is>
-      </c>
-      <c r="C88" t="inlineStr">
-        <is>
-          <t>Carmignac Flexible Bond A EUR Minc</t>
-        </is>
-      </c>
-      <c r="D88" t="inlineStr">
-        <is>
-          <t>Carmignac</t>
-        </is>
-      </c>
-      <c r="E88" t="inlineStr">
-        <is>
-          <t>Obb. Misti</t>
-        </is>
-      </c>
-      <c r="F88" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="G88" t="n">
-        <v>976.88</v>
-      </c>
-      <c r="H88" t="n">
-        <v>977.7005</v>
-      </c>
-      <c r="I88" t="n">
-        <v>38.06</v>
-      </c>
-      <c r="J88" s="1" t="inlineStr">
-        <is>
-          <t>HOLD</t>
-        </is>
-      </c>
-      <c r="K88" t="inlineStr">
-        <is>
-          <t>2026-02-26 19:47</t>
-        </is>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="B89" t="inlineStr">
-        <is>
-          <t>LU1317704135</t>
-        </is>
-      </c>
-      <c r="C89" t="inlineStr">
-        <is>
-          <t>Carmignac Long-Short Europ. Eqs E EUR Acc</t>
-        </is>
-      </c>
-      <c r="D89" t="inlineStr">
-        <is>
-          <t>Carmignac</t>
-        </is>
-      </c>
-      <c r="E89" t="inlineStr">
-        <is>
-          <t>Altri</t>
-        </is>
-      </c>
-      <c r="F89" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="G89" t="n">
-        <v>178.75</v>
-      </c>
-      <c r="H89" t="n">
-        <v>178.0845</v>
-      </c>
-      <c r="I89" t="n">
-        <v>58.8</v>
-      </c>
-      <c r="J89" s="1" t="inlineStr">
-        <is>
-          <t>HOLD</t>
-        </is>
-      </c>
-      <c r="K89" t="inlineStr">
         <is>
           <t>2026-02-26 19:47</t>
         </is>
@@ -4762,7 +4676,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M19"/>
+  <dimension ref="A1:M21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5125,6 +5039,112 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>3</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>FR0010149302</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Carmignac Emergents A EUR Acc</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Carmignac</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Altri</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>1650.0419921875</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>2026-02-26 19:47</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>Hang FT Markets</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>3</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>FR0011269349</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Carmignac Emergents A EUR Ydis</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Carmignac</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Azionari Paesi Emergenti</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>215.6589965820312</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>2026-02-26 19:47</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>Hang FT Markets</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix: rimuovi Carmignac Sécurité AW Cap+Ydis da watchlist (hang FT Markets)
FR0010149120 - Carmignac Sécurité AW Cap EUR
FR0011269083 - Carmignac Sécurité AW EUR Ydis
Totale fondi watchlist: 84

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fondi_monitoraggio.xlsx
+++ b/fondi_monitoraggio.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K87"/>
+  <dimension ref="A1:K85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -543,7 +543,7 @@
       <c r="I2" t="n">
         <v>71.08</v>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
@@ -592,7 +592,7 @@
       <c r="I3" t="n">
         <v>69.92</v>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
@@ -641,7 +641,7 @@
       <c r="I4" t="n">
         <v>70.58</v>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
@@ -690,7 +690,7 @@
       <c r="I5" t="n">
         <v>70.08</v>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
@@ -739,7 +739,7 @@
       <c r="I6" t="n">
         <v>49.53</v>
       </c>
-      <c r="J6" s="1" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -788,7 +788,7 @@
       <c r="I7" t="n">
         <v>6.63</v>
       </c>
-      <c r="J7" s="1" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -837,7 +837,7 @@
       <c r="I8" t="n">
         <v>74.39</v>
       </c>
-      <c r="J8" s="3" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>SELL</t>
         </is>
@@ -886,7 +886,7 @@
       <c r="I9" t="n">
         <v>78.56</v>
       </c>
-      <c r="J9" s="3" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>SELL</t>
         </is>
@@ -935,7 +935,7 @@
       <c r="I10" t="n">
         <v>76.48999999999999</v>
       </c>
-      <c r="J10" s="3" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>SELL</t>
         </is>
@@ -984,7 +984,7 @@
       <c r="I11" t="n">
         <v>68.19</v>
       </c>
-      <c r="J11" s="3" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>SELL</t>
         </is>
@@ -1033,7 +1033,7 @@
       <c r="I12" t="n">
         <v>74.66</v>
       </c>
-      <c r="J12" s="3" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>SELL</t>
         </is>
@@ -1082,7 +1082,7 @@
       <c r="I13" t="n">
         <v>64.3</v>
       </c>
-      <c r="J13" s="1" t="inlineStr">
+      <c r="J13" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -1094,7 +1094,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="n">
+      <c r="A14" t="n">
         <v>2</v>
       </c>
       <c r="B14" t="inlineStr">
@@ -1131,7 +1131,7 @@
       <c r="I14" t="n">
         <v>62.47</v>
       </c>
-      <c r="J14" s="1" t="inlineStr">
+      <c r="J14" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -1180,7 +1180,7 @@
       <c r="I15" t="n">
         <v>55.14</v>
       </c>
-      <c r="J15" s="1" t="inlineStr">
+      <c r="J15" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -1229,7 +1229,7 @@
       <c r="I16" t="n">
         <v>52.97</v>
       </c>
-      <c r="J16" s="1" t="inlineStr">
+      <c r="J16" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -1278,7 +1278,7 @@
       <c r="I17" t="n">
         <v>55.4</v>
       </c>
-      <c r="J17" s="1" t="inlineStr">
+      <c r="J17" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -1327,7 +1327,7 @@
       <c r="I18" t="n">
         <v>55</v>
       </c>
-      <c r="J18" s="1" t="inlineStr">
+      <c r="J18" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -1376,7 +1376,7 @@
       <c r="I19" t="n">
         <v>72.56999999999999</v>
       </c>
-      <c r="J19" s="3" t="inlineStr">
+      <c r="J19" t="inlineStr">
         <is>
           <t>SELL</t>
         </is>
@@ -1425,7 +1425,7 @@
       <c r="I20" t="n">
         <v>69.73999999999999</v>
       </c>
-      <c r="J20" s="1" t="inlineStr">
+      <c r="J20" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -1474,7 +1474,7 @@
       <c r="I21" t="n">
         <v>61.47</v>
       </c>
-      <c r="J21" s="1" t="inlineStr">
+      <c r="J21" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -1523,7 +1523,7 @@
       <c r="I22" t="n">
         <v>55.77</v>
       </c>
-      <c r="J22" s="1" t="inlineStr">
+      <c r="J22" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -1535,7 +1535,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="n">
+      <c r="A23" t="n">
         <v>2</v>
       </c>
       <c r="B23" t="inlineStr">
@@ -1572,7 +1572,7 @@
       <c r="I23" t="n">
         <v>57.83</v>
       </c>
-      <c r="J23" s="1" t="inlineStr">
+      <c r="J23" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -1621,7 +1621,7 @@
       <c r="I24" t="n">
         <v>73.44</v>
       </c>
-      <c r="J24" s="1" t="inlineStr">
+      <c r="J24" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -1633,7 +1633,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="n">
+      <c r="A25" t="n">
         <v>2</v>
       </c>
       <c r="B25" t="inlineStr">
@@ -1670,7 +1670,7 @@
       <c r="I25" t="n">
         <v>73.91</v>
       </c>
-      <c r="J25" s="2" t="inlineStr">
+      <c r="J25" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
@@ -1719,7 +1719,7 @@
       <c r="I26" t="n">
         <v>54.83</v>
       </c>
-      <c r="J26" s="1" t="inlineStr">
+      <c r="J26" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -1768,7 +1768,7 @@
       <c r="I27" t="n">
         <v>70.31</v>
       </c>
-      <c r="J27" s="1" t="inlineStr">
+      <c r="J27" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -1817,7 +1817,7 @@
       <c r="I28" t="n">
         <v>81.16</v>
       </c>
-      <c r="J28" s="2" t="inlineStr">
+      <c r="J28" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
@@ -1866,7 +1866,7 @@
       <c r="I29" t="n">
         <v>55.28</v>
       </c>
-      <c r="J29" s="1" t="inlineStr">
+      <c r="J29" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -1915,7 +1915,7 @@
       <c r="I30" t="n">
         <v>50.14</v>
       </c>
-      <c r="J30" s="1" t="inlineStr">
+      <c r="J30" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -1927,7 +1927,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="4" t="n">
+      <c r="A31" t="n">
         <v>3</v>
       </c>
       <c r="B31" t="inlineStr">
@@ -1964,7 +1964,7 @@
       <c r="I31" t="n">
         <v>35.5</v>
       </c>
-      <c r="J31" s="1" t="inlineStr">
+      <c r="J31" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -2013,7 +2013,7 @@
       <c r="I32" t="n">
         <v>68.95</v>
       </c>
-      <c r="J32" s="1" t="inlineStr">
+      <c r="J32" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -2056,7 +2056,7 @@
       <c r="G33" t="n">
         <v>72.44599914550781</v>
       </c>
-      <c r="J33" s="1" t="inlineStr">
+      <c r="J33" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -2068,7 +2068,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="4" t="n">
+      <c r="A34" t="n">
         <v>3</v>
       </c>
       <c r="B34" t="inlineStr">
@@ -2105,7 +2105,7 @@
       <c r="I34" t="n">
         <v>62.64</v>
       </c>
-      <c r="J34" s="1" t="inlineStr">
+      <c r="J34" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -2154,7 +2154,7 @@
       <c r="I35" t="n">
         <v>58.56</v>
       </c>
-      <c r="J35" s="1" t="inlineStr">
+      <c r="J35" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -2166,7 +2166,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="4" t="n">
+      <c r="A36" t="n">
         <v>3</v>
       </c>
       <c r="B36" t="inlineStr">
@@ -2203,7 +2203,7 @@
       <c r="I36" t="n">
         <v>45.48</v>
       </c>
-      <c r="J36" s="1" t="inlineStr">
+      <c r="J36" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -2246,7 +2246,7 @@
       <c r="G37" t="n">
         <v>12.55599975585938</v>
       </c>
-      <c r="J37" s="1" t="inlineStr">
+      <c r="J37" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -2258,7 +2258,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="4" t="n">
+      <c r="A38" t="n">
         <v>3</v>
       </c>
       <c r="B38" t="inlineStr">
@@ -2295,7 +2295,7 @@
       <c r="I38" t="n">
         <v>63.5</v>
       </c>
-      <c r="J38" s="1" t="inlineStr">
+      <c r="J38" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -2344,7 +2344,7 @@
       <c r="I39" t="n">
         <v>36.64</v>
       </c>
-      <c r="J39" s="1" t="inlineStr">
+      <c r="J39" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -2393,7 +2393,7 @@
       <c r="I40" t="n">
         <v>70.62</v>
       </c>
-      <c r="J40" s="1" t="inlineStr">
+      <c r="J40" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -2442,7 +2442,7 @@
       <c r="I41" t="n">
         <v>100</v>
       </c>
-      <c r="J41" s="1" t="inlineStr">
+      <c r="J41" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -2491,7 +2491,7 @@
       <c r="I42" t="n">
         <v>76.47</v>
       </c>
-      <c r="J42" s="1" t="inlineStr">
+      <c r="J42" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -2540,7 +2540,7 @@
       <c r="I43" t="n">
         <v>73.76000000000001</v>
       </c>
-      <c r="J43" s="1" t="inlineStr">
+      <c r="J43" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -2589,7 +2589,7 @@
       <c r="I44" t="n">
         <v>100</v>
       </c>
-      <c r="J44" s="1" t="inlineStr">
+      <c r="J44" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -2638,7 +2638,7 @@
       <c r="I45" t="n">
         <v>70.97</v>
       </c>
-      <c r="J45" s="1" t="inlineStr">
+      <c r="J45" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -2687,7 +2687,7 @@
       <c r="I46" t="n">
         <v>67.95999999999999</v>
       </c>
-      <c r="J46" s="1" t="inlineStr">
+      <c r="J46" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -2736,7 +2736,7 @@
       <c r="I47" t="n">
         <v>88.51000000000001</v>
       </c>
-      <c r="J47" s="1" t="inlineStr">
+      <c r="J47" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -2785,7 +2785,7 @@
       <c r="I48" t="n">
         <v>87.31</v>
       </c>
-      <c r="J48" s="1" t="inlineStr">
+      <c r="J48" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -2834,7 +2834,7 @@
       <c r="I49" t="n">
         <v>68.13</v>
       </c>
-      <c r="J49" s="1" t="inlineStr">
+      <c r="J49" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -2883,7 +2883,7 @@
       <c r="I50" t="n">
         <v>55.18</v>
       </c>
-      <c r="J50" s="1" t="inlineStr">
+      <c r="J50" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -2932,7 +2932,7 @@
       <c r="I51" t="n">
         <v>68.39</v>
       </c>
-      <c r="J51" s="1" t="inlineStr">
+      <c r="J51" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -2981,7 +2981,7 @@
       <c r="I52" t="n">
         <v>51.08</v>
       </c>
-      <c r="J52" s="1" t="inlineStr">
+      <c r="J52" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -3030,7 +3030,7 @@
       <c r="I53" t="n">
         <v>59.83</v>
       </c>
-      <c r="J53" s="1" t="inlineStr">
+      <c r="J53" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -3079,7 +3079,7 @@
       <c r="I54" t="n">
         <v>79.70999999999999</v>
       </c>
-      <c r="J54" s="1" t="inlineStr">
+      <c r="J54" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -3128,7 +3128,7 @@
       <c r="I55" t="n">
         <v>57.17</v>
       </c>
-      <c r="J55" s="1" t="inlineStr">
+      <c r="J55" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -3177,7 +3177,7 @@
       <c r="I56" t="n">
         <v>62.67</v>
       </c>
-      <c r="J56" s="1" t="inlineStr">
+      <c r="J56" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -3226,7 +3226,7 @@
       <c r="I57" t="n">
         <v>58.25</v>
       </c>
-      <c r="J57" s="1" t="inlineStr">
+      <c r="J57" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -3275,7 +3275,7 @@
       <c r="I58" t="n">
         <v>64.09999999999999</v>
       </c>
-      <c r="J58" s="1" t="inlineStr">
+      <c r="J58" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -3324,7 +3324,7 @@
       <c r="I59" t="n">
         <v>57.58</v>
       </c>
-      <c r="J59" s="1" t="inlineStr">
+      <c r="J59" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -3373,7 +3373,7 @@
       <c r="I60" t="n">
         <v>96.48999999999999</v>
       </c>
-      <c r="J60" s="1" t="inlineStr">
+      <c r="J60" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -3422,7 +3422,7 @@
       <c r="I61" t="n">
         <v>81.06</v>
       </c>
-      <c r="J61" s="1" t="inlineStr">
+      <c r="J61" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -3471,7 +3471,7 @@
       <c r="I62" t="n">
         <v>64.94</v>
       </c>
-      <c r="J62" s="1" t="inlineStr">
+      <c r="J62" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -3520,7 +3520,7 @@
       <c r="I63" t="n">
         <v>63.81</v>
       </c>
-      <c r="J63" s="1" t="inlineStr">
+      <c r="J63" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -3569,7 +3569,7 @@
       <c r="I64" t="n">
         <v>62.06</v>
       </c>
-      <c r="J64" s="1" t="inlineStr">
+      <c r="J64" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -3618,7 +3618,7 @@
       <c r="I65" t="n">
         <v>71.58</v>
       </c>
-      <c r="J65" s="1" t="inlineStr">
+      <c r="J65" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -3667,7 +3667,7 @@
       <c r="I66" t="n">
         <v>71.15000000000001</v>
       </c>
-      <c r="J66" s="1" t="inlineStr">
+      <c r="J66" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -3716,7 +3716,7 @@
       <c r="I67" t="n">
         <v>69.03</v>
       </c>
-      <c r="J67" s="1" t="inlineStr">
+      <c r="J67" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -3765,7 +3765,7 @@
       <c r="I68" t="n">
         <v>71.95999999999999</v>
       </c>
-      <c r="J68" s="1" t="inlineStr">
+      <c r="J68" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -3814,7 +3814,7 @@
       <c r="I69" t="n">
         <v>77.36</v>
       </c>
-      <c r="J69" s="1" t="inlineStr">
+      <c r="J69" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -3863,7 +3863,7 @@
       <c r="I70" t="n">
         <v>30.23</v>
       </c>
-      <c r="J70" s="1" t="inlineStr">
+      <c r="J70" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -3912,7 +3912,7 @@
       <c r="I71" t="n">
         <v>54.93</v>
       </c>
-      <c r="J71" s="1" t="inlineStr">
+      <c r="J71" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -3961,7 +3961,7 @@
       <c r="I72" t="n">
         <v>46.8</v>
       </c>
-      <c r="J72" s="1" t="inlineStr">
+      <c r="J72" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -3978,12 +3978,12 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>FR0010149120</t>
+          <t>FR0010312660</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Carmignac Sécurité AW Cap EUR</t>
+          <t>Carmignac Investissement E EUR Acc</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -3993,7 +3993,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Obb. Misti</t>
+          <t>Altri</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -4002,9 +4002,15 @@
         </is>
       </c>
       <c r="G73" t="n">
-        <v>1926.787963867188</v>
-      </c>
-      <c r="J73" s="1" t="inlineStr">
+        <v>355.64</v>
+      </c>
+      <c r="H73" t="n">
+        <v>348.33</v>
+      </c>
+      <c r="I73" t="n">
+        <v>61.47</v>
+      </c>
+      <c r="J73" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -4021,12 +4027,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>FR0010312660</t>
+          <t>LU0336083810</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Carmignac Investissement E EUR Acc</t>
+          <t>Carmignac Asia Discovery A EUR Acc EUR</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -4036,7 +4042,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Altri</t>
+          <t>Azionari Paesi Emergenti</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -4045,15 +4051,9 @@
         </is>
       </c>
       <c r="G74" t="n">
-        <v>355.64</v>
-      </c>
-      <c r="H74" t="n">
-        <v>348.33</v>
-      </c>
-      <c r="I74" t="n">
-        <v>61.47</v>
-      </c>
-      <c r="J74" s="1" t="inlineStr">
+        <v>2717.27099609375</v>
+      </c>
+      <c r="J74" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -4066,16 +4066,16 @@
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>LU0336083810</t>
+          <t>FR0011269182</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Carmignac Asia Discovery A EUR Acc EUR</t>
+          <t>Carmignac Investissement A EUR Ydis</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -4085,7 +4085,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Azionari Paesi Emergenti</t>
+          <t>Azionari Internazionali</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -4094,9 +4094,15 @@
         </is>
       </c>
       <c r="G75" t="n">
-        <v>2717.27099609375</v>
-      </c>
-      <c r="J75" s="1" t="inlineStr">
+        <v>279.91</v>
+      </c>
+      <c r="H75" t="n">
+        <v>278.601</v>
+      </c>
+      <c r="I75" t="n">
+        <v>47.36</v>
+      </c>
+      <c r="J75" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -4108,17 +4114,17 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="2" t="n">
+      <c r="A76" t="n">
         <v>2</v>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>FR0011269182</t>
+          <t>LU1317704051</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Carmignac Investissement A EUR Ydis</t>
+          <t>Carmignac Long-Short Europ. Eqs A EUR Acc</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -4128,7 +4134,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Azionari Internazionali</t>
+          <t>Altri</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -4137,15 +4143,15 @@
         </is>
       </c>
       <c r="G76" t="n">
-        <v>279.91</v>
+        <v>190.63</v>
       </c>
       <c r="H76" t="n">
-        <v>278.601</v>
+        <v>189.8945</v>
       </c>
       <c r="I76" t="n">
-        <v>47.36</v>
-      </c>
-      <c r="J76" s="1" t="inlineStr">
+        <v>59.29</v>
+      </c>
+      <c r="J76" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -4162,12 +4168,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>FR0011269083</t>
+          <t>LU1163533349</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Carmignac Sécurité AW EUR Ydis</t>
+          <t>Carmignac Patrimoine E EUR Minc</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -4177,7 +4183,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Fondi Flessibili</t>
+          <t>Altri</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -4186,9 +4192,15 @@
         </is>
       </c>
       <c r="G77" t="n">
-        <v>99.56800079345703</v>
-      </c>
-      <c r="J77" s="1" t="inlineStr">
+        <v>69.37</v>
+      </c>
+      <c r="H77" t="n">
+        <v>68.967</v>
+      </c>
+      <c r="I77" t="n">
+        <v>54.11</v>
+      </c>
+      <c r="J77" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -4200,17 +4212,17 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="4" t="n">
-        <v>2</v>
+      <c r="A78" t="n">
+        <v>3</v>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>LU1317704051</t>
+          <t>FR0011269588</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Carmignac Long-Short Europ. Eqs A EUR Acc</t>
+          <t>Carmignac Patrimoine A EUR Ydis</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -4220,7 +4232,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Altri</t>
+          <t>Bilanciati</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -4229,15 +4241,9 @@
         </is>
       </c>
       <c r="G78" t="n">
-        <v>190.63</v>
-      </c>
-      <c r="H78" t="n">
-        <v>189.8945</v>
-      </c>
-      <c r="I78" t="n">
-        <v>59.29</v>
-      </c>
-      <c r="J78" s="1" t="inlineStr">
+        <v>128.2530059814453</v>
+      </c>
+      <c r="J78" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -4254,12 +4260,12 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>LU1163533349</t>
+          <t>LU1163533422</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Carmignac Patrimoine E EUR Minc</t>
+          <t>Carmignac Patrimoine A EUR Minc</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -4278,15 +4284,15 @@
         </is>
       </c>
       <c r="G79" t="n">
-        <v>69.37</v>
+        <v>73.19</v>
       </c>
       <c r="H79" t="n">
-        <v>68.967</v>
+        <v>72.76049999999999</v>
       </c>
       <c r="I79" t="n">
-        <v>54.11</v>
-      </c>
-      <c r="J79" s="1" t="inlineStr">
+        <v>54.86</v>
+      </c>
+      <c r="J79" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -4303,12 +4309,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>FR0011269588</t>
+          <t>FR0010135103</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Carmignac Patrimoine A EUR Ydis</t>
+          <t>Carmignac Patrimoine A EUR Acc</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -4327,9 +4333,9 @@
         </is>
       </c>
       <c r="G80" t="n">
-        <v>128.2530059814453</v>
-      </c>
-      <c r="J80" s="1" t="inlineStr">
+        <v>800.5250244140625</v>
+      </c>
+      <c r="J80" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -4346,12 +4352,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>LU1163533422</t>
+          <t>FR0010306142</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Carmignac Patrimoine A EUR Minc</t>
+          <t>Carmignac Patrimoine E EUR Acc</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -4361,7 +4367,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Altri</t>
+          <t>Bilanciati</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -4370,15 +4376,15 @@
         </is>
       </c>
       <c r="G81" t="n">
-        <v>73.19</v>
+        <v>192.75</v>
       </c>
       <c r="H81" t="n">
-        <v>72.76049999999999</v>
+        <v>191.6865</v>
       </c>
       <c r="I81" t="n">
-        <v>54.86</v>
-      </c>
-      <c r="J81" s="1" t="inlineStr">
+        <v>57.09</v>
+      </c>
+      <c r="J81" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -4395,12 +4401,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>FR0010135103</t>
+          <t>LU0336084032</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Carmignac Patrimoine A EUR Acc</t>
+          <t>Carmignac Flexible Bond A EUR Acc</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -4410,7 +4416,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Bilanciati</t>
+          <t>Obb. Misti</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -4419,9 +4425,9 @@
         </is>
       </c>
       <c r="G82" t="n">
-        <v>800.5250244140625</v>
-      </c>
-      <c r="J82" s="1" t="inlineStr">
+        <v>1380.400024414062</v>
+      </c>
+      <c r="J82" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -4438,12 +4444,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>FR0010306142</t>
+          <t>LU0992631050</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Carmignac Patrimoine E EUR Acc</t>
+          <t>Carmignac Flexible Bond A EUR Ydis</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -4453,7 +4459,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Bilanciati</t>
+          <t>Obb. Misti</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -4462,15 +4468,9 @@
         </is>
       </c>
       <c r="G83" t="n">
-        <v>192.75</v>
-      </c>
-      <c r="H83" t="n">
-        <v>191.6865</v>
-      </c>
-      <c r="I83" t="n">
-        <v>57.09</v>
-      </c>
-      <c r="J83" s="1" t="inlineStr">
+        <v>1090.800048828125</v>
+      </c>
+      <c r="J83" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -4487,12 +4487,12 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>LU0336084032</t>
+          <t>LU1299302684</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Carmignac Flexible Bond A EUR Acc</t>
+          <t>Carmignac Flexible Bond A EUR Minc</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -4511,9 +4511,15 @@
         </is>
       </c>
       <c r="G84" t="n">
-        <v>1380.400024414062</v>
-      </c>
-      <c r="J84" s="1" t="inlineStr">
+        <v>976.88</v>
+      </c>
+      <c r="H84" t="n">
+        <v>977.7005</v>
+      </c>
+      <c r="I84" t="n">
+        <v>38.06</v>
+      </c>
+      <c r="J84" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -4526,16 +4532,16 @@
     </row>
     <row r="85">
       <c r="A85" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>LU0992631050</t>
+          <t>LU1317704135</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Carmignac Flexible Bond A EUR Ydis</t>
+          <t>Carmignac Long-Short Europ. Eqs E EUR Acc</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -4545,7 +4551,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Obb. Misti</t>
+          <t>Altri</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -4554,112 +4560,20 @@
         </is>
       </c>
       <c r="G85" t="n">
-        <v>1090.800048828125</v>
-      </c>
-      <c r="J85" s="1" t="inlineStr">
+        <v>178.75</v>
+      </c>
+      <c r="H85" t="n">
+        <v>178.0845</v>
+      </c>
+      <c r="I85" t="n">
+        <v>58.8</v>
+      </c>
+      <c r="J85" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
       </c>
       <c r="K85" t="inlineStr">
-        <is>
-          <t>2026-02-26 19:47</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" t="n">
-        <v>3</v>
-      </c>
-      <c r="B86" t="inlineStr">
-        <is>
-          <t>LU1299302684</t>
-        </is>
-      </c>
-      <c r="C86" t="inlineStr">
-        <is>
-          <t>Carmignac Flexible Bond A EUR Minc</t>
-        </is>
-      </c>
-      <c r="D86" t="inlineStr">
-        <is>
-          <t>Carmignac</t>
-        </is>
-      </c>
-      <c r="E86" t="inlineStr">
-        <is>
-          <t>Obb. Misti</t>
-        </is>
-      </c>
-      <c r="F86" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="G86" t="n">
-        <v>976.88</v>
-      </c>
-      <c r="H86" t="n">
-        <v>977.7005</v>
-      </c>
-      <c r="I86" t="n">
-        <v>38.06</v>
-      </c>
-      <c r="J86" s="1" t="inlineStr">
-        <is>
-          <t>HOLD</t>
-        </is>
-      </c>
-      <c r="K86" t="inlineStr">
-        <is>
-          <t>2026-02-26 19:47</t>
-        </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="B87" t="inlineStr">
-        <is>
-          <t>LU1317704135</t>
-        </is>
-      </c>
-      <c r="C87" t="inlineStr">
-        <is>
-          <t>Carmignac Long-Short Europ. Eqs E EUR Acc</t>
-        </is>
-      </c>
-      <c r="D87" t="inlineStr">
-        <is>
-          <t>Carmignac</t>
-        </is>
-      </c>
-      <c r="E87" t="inlineStr">
-        <is>
-          <t>Altri</t>
-        </is>
-      </c>
-      <c r="F87" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="G87" t="n">
-        <v>178.75</v>
-      </c>
-      <c r="H87" t="n">
-        <v>178.0845</v>
-      </c>
-      <c r="I87" t="n">
-        <v>58.8</v>
-      </c>
-      <c r="J87" s="1" t="inlineStr">
-        <is>
-          <t>HOLD</t>
-        </is>
-      </c>
-      <c r="K87" t="inlineStr">
         <is>
           <t>2026-02-26 19:47</t>
         </is>
@@ -4676,7 +4590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M21"/>
+  <dimension ref="A1:M23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5145,6 +5059,92 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>3</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>FR0010149120</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Carmignac Sécurité AW Cap EUR</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Carmignac</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Obb. Misti</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
+        <v>1926.787963867188</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>2026-02-26 19:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>3</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>FR0011269083</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Carmignac Sécurité AW EUR Ydis</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Carmignac</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Fondi Flessibili</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>99.56800079345703</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>2026-02-26 19:47</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix: rimuovi Carmignac Patrimoine/FlexBond/LongShortE (hang FT Markets)
9 fondi rimossi (Patrimoine x5, Flexible Bond x3, Long-Short E x1)
Fondi watchlist: 75

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fondi_monitoraggio.xlsx
+++ b/fondi_monitoraggio.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K85"/>
+  <dimension ref="A1:K76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4157,423 +4157,6 @@
         </is>
       </c>
       <c r="K76" t="inlineStr">
-        <is>
-          <t>2026-02-26 19:47</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" t="n">
-        <v>3</v>
-      </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>LU1163533349</t>
-        </is>
-      </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>Carmignac Patrimoine E EUR Minc</t>
-        </is>
-      </c>
-      <c r="D77" t="inlineStr">
-        <is>
-          <t>Carmignac</t>
-        </is>
-      </c>
-      <c r="E77" t="inlineStr">
-        <is>
-          <t>Altri</t>
-        </is>
-      </c>
-      <c r="F77" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="G77" t="n">
-        <v>69.37</v>
-      </c>
-      <c r="H77" t="n">
-        <v>68.967</v>
-      </c>
-      <c r="I77" t="n">
-        <v>54.11</v>
-      </c>
-      <c r="J77" t="inlineStr">
-        <is>
-          <t>HOLD</t>
-        </is>
-      </c>
-      <c r="K77" t="inlineStr">
-        <is>
-          <t>2026-02-26 19:47</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" t="n">
-        <v>3</v>
-      </c>
-      <c r="B78" t="inlineStr">
-        <is>
-          <t>FR0011269588</t>
-        </is>
-      </c>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>Carmignac Patrimoine A EUR Ydis</t>
-        </is>
-      </c>
-      <c r="D78" t="inlineStr">
-        <is>
-          <t>Carmignac</t>
-        </is>
-      </c>
-      <c r="E78" t="inlineStr">
-        <is>
-          <t>Bilanciati</t>
-        </is>
-      </c>
-      <c r="F78" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="G78" t="n">
-        <v>128.2530059814453</v>
-      </c>
-      <c r="J78" t="inlineStr">
-        <is>
-          <t>HOLD</t>
-        </is>
-      </c>
-      <c r="K78" t="inlineStr">
-        <is>
-          <t>2026-02-26 19:47</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" t="n">
-        <v>3</v>
-      </c>
-      <c r="B79" t="inlineStr">
-        <is>
-          <t>LU1163533422</t>
-        </is>
-      </c>
-      <c r="C79" t="inlineStr">
-        <is>
-          <t>Carmignac Patrimoine A EUR Minc</t>
-        </is>
-      </c>
-      <c r="D79" t="inlineStr">
-        <is>
-          <t>Carmignac</t>
-        </is>
-      </c>
-      <c r="E79" t="inlineStr">
-        <is>
-          <t>Altri</t>
-        </is>
-      </c>
-      <c r="F79" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="G79" t="n">
-        <v>73.19</v>
-      </c>
-      <c r="H79" t="n">
-        <v>72.76049999999999</v>
-      </c>
-      <c r="I79" t="n">
-        <v>54.86</v>
-      </c>
-      <c r="J79" t="inlineStr">
-        <is>
-          <t>HOLD</t>
-        </is>
-      </c>
-      <c r="K79" t="inlineStr">
-        <is>
-          <t>2026-02-26 19:47</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" t="n">
-        <v>3</v>
-      </c>
-      <c r="B80" t="inlineStr">
-        <is>
-          <t>FR0010135103</t>
-        </is>
-      </c>
-      <c r="C80" t="inlineStr">
-        <is>
-          <t>Carmignac Patrimoine A EUR Acc</t>
-        </is>
-      </c>
-      <c r="D80" t="inlineStr">
-        <is>
-          <t>Carmignac</t>
-        </is>
-      </c>
-      <c r="E80" t="inlineStr">
-        <is>
-          <t>Bilanciati</t>
-        </is>
-      </c>
-      <c r="F80" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="G80" t="n">
-        <v>800.5250244140625</v>
-      </c>
-      <c r="J80" t="inlineStr">
-        <is>
-          <t>HOLD</t>
-        </is>
-      </c>
-      <c r="K80" t="inlineStr">
-        <is>
-          <t>2026-02-26 19:47</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" t="n">
-        <v>3</v>
-      </c>
-      <c r="B81" t="inlineStr">
-        <is>
-          <t>FR0010306142</t>
-        </is>
-      </c>
-      <c r="C81" t="inlineStr">
-        <is>
-          <t>Carmignac Patrimoine E EUR Acc</t>
-        </is>
-      </c>
-      <c r="D81" t="inlineStr">
-        <is>
-          <t>Carmignac</t>
-        </is>
-      </c>
-      <c r="E81" t="inlineStr">
-        <is>
-          <t>Bilanciati</t>
-        </is>
-      </c>
-      <c r="F81" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="G81" t="n">
-        <v>192.75</v>
-      </c>
-      <c r="H81" t="n">
-        <v>191.6865</v>
-      </c>
-      <c r="I81" t="n">
-        <v>57.09</v>
-      </c>
-      <c r="J81" t="inlineStr">
-        <is>
-          <t>HOLD</t>
-        </is>
-      </c>
-      <c r="K81" t="inlineStr">
-        <is>
-          <t>2026-02-26 19:47</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" t="n">
-        <v>3</v>
-      </c>
-      <c r="B82" t="inlineStr">
-        <is>
-          <t>LU0336084032</t>
-        </is>
-      </c>
-      <c r="C82" t="inlineStr">
-        <is>
-          <t>Carmignac Flexible Bond A EUR Acc</t>
-        </is>
-      </c>
-      <c r="D82" t="inlineStr">
-        <is>
-          <t>Carmignac</t>
-        </is>
-      </c>
-      <c r="E82" t="inlineStr">
-        <is>
-          <t>Obb. Misti</t>
-        </is>
-      </c>
-      <c r="F82" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="G82" t="n">
-        <v>1380.400024414062</v>
-      </c>
-      <c r="J82" t="inlineStr">
-        <is>
-          <t>HOLD</t>
-        </is>
-      </c>
-      <c r="K82" t="inlineStr">
-        <is>
-          <t>2026-02-26 19:47</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" t="n">
-        <v>3</v>
-      </c>
-      <c r="B83" t="inlineStr">
-        <is>
-          <t>LU0992631050</t>
-        </is>
-      </c>
-      <c r="C83" t="inlineStr">
-        <is>
-          <t>Carmignac Flexible Bond A EUR Ydis</t>
-        </is>
-      </c>
-      <c r="D83" t="inlineStr">
-        <is>
-          <t>Carmignac</t>
-        </is>
-      </c>
-      <c r="E83" t="inlineStr">
-        <is>
-          <t>Obb. Misti</t>
-        </is>
-      </c>
-      <c r="F83" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="G83" t="n">
-        <v>1090.800048828125</v>
-      </c>
-      <c r="J83" t="inlineStr">
-        <is>
-          <t>HOLD</t>
-        </is>
-      </c>
-      <c r="K83" t="inlineStr">
-        <is>
-          <t>2026-02-26 19:47</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" t="n">
-        <v>3</v>
-      </c>
-      <c r="B84" t="inlineStr">
-        <is>
-          <t>LU1299302684</t>
-        </is>
-      </c>
-      <c r="C84" t="inlineStr">
-        <is>
-          <t>Carmignac Flexible Bond A EUR Minc</t>
-        </is>
-      </c>
-      <c r="D84" t="inlineStr">
-        <is>
-          <t>Carmignac</t>
-        </is>
-      </c>
-      <c r="E84" t="inlineStr">
-        <is>
-          <t>Obb. Misti</t>
-        </is>
-      </c>
-      <c r="F84" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="G84" t="n">
-        <v>976.88</v>
-      </c>
-      <c r="H84" t="n">
-        <v>977.7005</v>
-      </c>
-      <c r="I84" t="n">
-        <v>38.06</v>
-      </c>
-      <c r="J84" t="inlineStr">
-        <is>
-          <t>HOLD</t>
-        </is>
-      </c>
-      <c r="K84" t="inlineStr">
-        <is>
-          <t>2026-02-26 19:47</t>
-        </is>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" t="n">
-        <v>2</v>
-      </c>
-      <c r="B85" t="inlineStr">
-        <is>
-          <t>LU1317704135</t>
-        </is>
-      </c>
-      <c r="C85" t="inlineStr">
-        <is>
-          <t>Carmignac Long-Short Europ. Eqs E EUR Acc</t>
-        </is>
-      </c>
-      <c r="D85" t="inlineStr">
-        <is>
-          <t>Carmignac</t>
-        </is>
-      </c>
-      <c r="E85" t="inlineStr">
-        <is>
-          <t>Altri</t>
-        </is>
-      </c>
-      <c r="F85" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="G85" t="n">
-        <v>178.75</v>
-      </c>
-      <c r="H85" t="n">
-        <v>178.0845</v>
-      </c>
-      <c r="I85" t="n">
-        <v>58.8</v>
-      </c>
-      <c r="J85" t="inlineStr">
-        <is>
-          <t>HOLD</t>
-        </is>
-      </c>
-      <c r="K85" t="inlineStr">
         <is>
           <t>2026-02-26 19:47</t>
         </is>
@@ -4590,7 +4173,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M23"/>
+  <dimension ref="A1:M32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5145,6 +4728,423 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>3</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>LU1163533349</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Carmignac Patrimoine E EUR Minc</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Carmignac</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Altri</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G24" t="n">
+        <v>69.37</v>
+      </c>
+      <c r="H24" t="n">
+        <v>68.967</v>
+      </c>
+      <c r="I24" t="n">
+        <v>54.11</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>2026-02-26 19:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>3</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>FR0011269588</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Carmignac Patrimoine A EUR Ydis</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Carmignac</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Bilanciati</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G25" t="n">
+        <v>128.2530059814453</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>2026-02-26 19:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>3</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>LU1163533422</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Carmignac Patrimoine A EUR Minc</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Carmignac</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Altri</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G26" t="n">
+        <v>73.19</v>
+      </c>
+      <c r="H26" t="n">
+        <v>72.76049999999999</v>
+      </c>
+      <c r="I26" t="n">
+        <v>54.86</v>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>2026-02-26 19:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>3</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>FR0010135103</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Carmignac Patrimoine A EUR Acc</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Carmignac</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Bilanciati</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G27" t="n">
+        <v>800.5250244140625</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>2026-02-26 19:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>3</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>FR0010306142</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Carmignac Patrimoine E EUR Acc</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Carmignac</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Bilanciati</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G28" t="n">
+        <v>192.75</v>
+      </c>
+      <c r="H28" t="n">
+        <v>191.6865</v>
+      </c>
+      <c r="I28" t="n">
+        <v>57.09</v>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>2026-02-26 19:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>3</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>LU0336084032</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Carmignac Flexible Bond A EUR Acc</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Carmignac</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Obb. Misti</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G29" t="n">
+        <v>1380.400024414062</v>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>2026-02-26 19:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>3</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>LU0992631050</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Carmignac Flexible Bond A EUR Ydis</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Carmignac</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Obb. Misti</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G30" t="n">
+        <v>1090.800048828125</v>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>2026-02-26 19:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>3</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>LU1299302684</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Carmignac Flexible Bond A EUR Minc</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Carmignac</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Obb. Misti</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G31" t="n">
+        <v>976.88</v>
+      </c>
+      <c r="H31" t="n">
+        <v>977.7005</v>
+      </c>
+      <c r="I31" t="n">
+        <v>38.06</v>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>2026-02-26 19:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>2</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>LU1317704135</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Carmignac Long-Short Europ. Eqs E EUR Acc</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Carmignac</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Altri</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G32" t="n">
+        <v>178.75</v>
+      </c>
+      <c r="H32" t="n">
+        <v>178.0845</v>
+      </c>
+      <c r="I32" t="n">
+        <v>58.8</v>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>2026-02-26 19:47</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Rimuovi Morgan Stanley EM (LU0073229840): dati non disponibili su FT Markets
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fondi_monitoraggio.xlsx
+++ b/fondi_monitoraggio.xlsx
@@ -384,7 +384,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:K103"/>
+  <dimension ref="A1:K102"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7578125" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="28.23" customWidth="1" style="5" min="2" max="2"/>
@@ -4504,7 +4504,7 @@
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="6">
-      <c r="A89" t="n">
+      <c r="A89" s="5" t="n">
         <v>3</v>
       </c>
       <c r="B89" s="8" t="inlineStr">
@@ -4537,7 +4537,7 @@
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="6">
-      <c r="A90" t="n">
+      <c r="A90" s="5" t="n">
         <v>3</v>
       </c>
       <c r="B90" s="8" t="inlineStr">
@@ -4570,7 +4570,7 @@
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="6">
-      <c r="A91" t="n">
+      <c r="A91" s="5" t="n">
         <v>3</v>
       </c>
       <c r="B91" s="8" t="inlineStr">
@@ -4603,7 +4603,7 @@
       </c>
     </row>
     <row r="92" ht="15" customHeight="1" s="6">
-      <c r="A92" t="n">
+      <c r="A92" s="5" t="n">
         <v>3</v>
       </c>
       <c r="B92" s="8" t="inlineStr">
@@ -4636,7 +4636,7 @@
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="6">
-      <c r="A93" t="n">
+      <c r="A93" s="5" t="n">
         <v>3</v>
       </c>
       <c r="B93" s="8" t="inlineStr">
@@ -4669,7 +4669,7 @@
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="6">
-      <c r="A94" t="n">
+      <c r="A94" s="5" t="n">
         <v>3</v>
       </c>
       <c r="B94" s="8" t="inlineStr">
@@ -4702,7 +4702,7 @@
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="6">
-      <c r="A95" t="n">
+      <c r="A95" s="5" t="n">
         <v>3</v>
       </c>
       <c r="B95" s="8" t="inlineStr">
@@ -4735,7 +4735,7 @@
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="6">
-      <c r="A96" t="n">
+      <c r="A96" s="5" t="n">
         <v>3</v>
       </c>
       <c r="B96" s="8" t="inlineStr">
@@ -4768,7 +4768,7 @@
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="6">
-      <c r="A97" t="n">
+      <c r="A97" s="5" t="n">
         <v>3</v>
       </c>
       <c r="B97" s="8" t="inlineStr">
@@ -4801,7 +4801,7 @@
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="6">
-      <c r="A98" t="n">
+      <c r="A98" s="5" t="n">
         <v>3</v>
       </c>
       <c r="B98" s="8" t="inlineStr">
@@ -4834,7 +4834,7 @@
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="6">
-      <c r="A99" t="n">
+      <c r="A99" s="5" t="n">
         <v>3</v>
       </c>
       <c r="B99" s="8" t="inlineStr">
@@ -4867,7 +4867,7 @@
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="6">
-      <c r="A100" t="n">
+      <c r="A100" s="5" t="n">
         <v>3</v>
       </c>
       <c r="B100" s="8" t="inlineStr">
@@ -4900,7 +4900,7 @@
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="6">
-      <c r="A101" t="n">
+      <c r="A101" s="5" t="n">
         <v>3</v>
       </c>
       <c r="B101" s="8" t="inlineStr">
@@ -4933,27 +4933,27 @@
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="6">
-      <c r="A102" t="n">
+      <c r="A102" s="5" t="n">
         <v>3</v>
       </c>
       <c r="B102" s="8" t="inlineStr">
         <is>
-          <t>LU0073229840</t>
+          <t>LU0300834669</t>
         </is>
       </c>
       <c r="C102" s="7" t="inlineStr">
         <is>
-          <t>Morgan Stanley Emerging Markets Equity Fund Classe A EUR Acc</t>
+          <t>Alken Fund - Small Cap Europe Eur Classe R</t>
         </is>
       </c>
       <c r="D102" s="8" t="inlineStr">
         <is>
-          <t>Morgan Stanley Investment Fund SICAV</t>
+          <t>Alken Fund SICAV</t>
         </is>
       </c>
       <c r="E102" s="8" t="inlineStr">
         <is>
-          <t>Azionari Globali (Mercati Emergenti) - Large &amp; Mid Cap Growth</t>
+          <t>Azionari Europa (Mercati Sviluppati) - Small Cap</t>
         </is>
       </c>
       <c r="F102" s="5" t="inlineStr">
@@ -4962,42 +4962,10 @@
         </is>
       </c>
       <c r="G102" s="8" t="n">
-        <v>62.97</v>
-      </c>
-    </row>
-    <row r="103" ht="15" customHeight="1" s="6">
-      <c r="A103" t="n">
-        <v>3</v>
-      </c>
-      <c r="B103" s="8" t="inlineStr">
-        <is>
-          <t>LU0300834669</t>
-        </is>
-      </c>
-      <c r="C103" s="7" t="inlineStr">
-        <is>
-          <t>Alken Fund - Small Cap Europe Eur Classe R</t>
-        </is>
-      </c>
-      <c r="D103" s="8" t="inlineStr">
-        <is>
-          <t>Alken Fund SICAV</t>
-        </is>
-      </c>
-      <c r="E103" s="8" t="inlineStr">
-        <is>
-          <t>Azionari Europa (Mercati Sviluppati) - Small Cap</t>
-        </is>
-      </c>
-      <c r="F103" s="5" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="G103" s="8" t="n">
         <v>607.48</v>
       </c>
     </row>
+    <row r="103" ht="15" customHeight="1" s="6"/>
     <row r="104" ht="15" customHeight="1" s="6"/>
     <row r="1048575" ht="12.75" customHeight="1" s="6"/>
     <row r="1048576" ht="12.8" customHeight="1" s="6"/>

</xml_diff>